<commit_message>
Update project time tracking through June 30
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\mechanical-technical-document-evaluation-harness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A521B76E-48B1-411C-A464-94AF8EAAD0B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E51EF632-F772-486E-AC30-B7656800CD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="994" uniqueCount="425">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="431">
   <si>
     <t>Mechanical Technical Document Evaluation Harness — Baseline Control Plan</t>
   </si>
@@ -499,9 +499,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>Not Started</t>
-  </si>
-  <si>
     <t>0.2</t>
   </si>
   <si>
@@ -527,6 +524,9 @@
   </si>
   <si>
     <t>Weekly review checklist and change-control rule</t>
+  </si>
+  <si>
+    <t>Not Started</t>
   </si>
   <si>
     <t>0.5</t>
@@ -1294,13 +1294,31 @@
     <t>Informs authentic mechanical document, QA/QC, revision, maintenance, and technical-record workflow selection.</t>
   </si>
   <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Completed before baseline start on 2026-06-28. Python 3.14.2 virtual environment active; baseline tests passed.</t>
+  </si>
+  <si>
+    <t>Completed 2026-06-30. Local Git initialized, baseline commit created, GitHub origin configured, and main pushed successfully. Actual time was not separately logged.</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>Complete</t>
+    <t>Repository layout, README, CLI commands, and MECH-001 summary reviewed. Full four-schema walkthrough and concise architecture explanation remain.</t>
   </si>
   <si>
-    <t>Done on Sun. 29 of June.</t>
+    <t>Week 1 control update completed. Actual time is recorded only where explicitly tracked.</t>
+  </si>
+  <si>
+    <t>Started early. Created feature/test-unknown-case and added the first controlled test change. Push/PR/merge evidence and two more branches plus recovery exercise remain.</t>
+  </si>
+  <si>
+    <t>Completed early on 2026-06-30. Added a negative CLI integration test; 20 tests pass locally. Actual time was not separately logged.</t>
+  </si>
+  <si>
+    <t>Completed Python environment and Git/GitHub baseline; validated all 3 seed cases; inspected MECH-001; reached 20 passing tests. Only 1.5 hours were explicitly time-tracked, so other completed work remains unallocated in Actual Hours.</t>
   </si>
 </sst>
 </file>
@@ -1866,6 +1884,30 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1893,15 +1935,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1909,21 +1942,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1942,7 +1960,7 @@
         <color rgb="FF166534"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
@@ -1952,7 +1970,7 @@
         <color rgb="FF991B1B"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
@@ -1962,7 +1980,7 @@
         <color rgb="FF166534"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
@@ -1972,7 +1990,7 @@
         <color rgb="FF991B1B"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
@@ -1983,7 +2001,7 @@
         <color rgb="FF991B1B"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFFEE2E2"/>
         </patternFill>
       </fill>
@@ -1994,7 +2012,7 @@
         <color rgb="FF1D4ED8"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFDBEAFE"/>
         </patternFill>
       </fill>
@@ -2005,7 +2023,7 @@
         <color rgb="FF166534"/>
       </font>
       <fill>
-        <patternFill patternType="solid">
+        <patternFill>
           <bgColor rgb="FFDCFCE7"/>
         </patternFill>
       </fill>
@@ -2375,7 +2393,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-767D-4A5B-9406-5124E6BCB77C}"/>
+              <c16:uniqueId val="{00000000-385B-41B8-85CE-A9C9AFF7D0EE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2556,13 +2574,16 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="52"/>
+                <c:pt idx="0">
+                  <c:v>1.5</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-767D-4A5B-9406-5124E6BCB77C}"/>
+              <c16:uniqueId val="{00000001-385B-41B8-85CE-A9C9AFF7D0EE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2671,7 +2692,6 @@
           <a:lstStyle/>
           <a:p>
             <a:r>
-              <a:rPr lang="en-US"/>
               <a:t>Planned Hours by Phase</a:t>
             </a:r>
           </a:p>
@@ -2760,7 +2780,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-BDD9-4EC5-962B-6A087F44F17F}"/>
+              <c16:uniqueId val="{00000000-E919-4C75-A1FE-46BAE985CCA2}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3137,16 +3157,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="30" customHeight="1">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -3288,13 +3308,13 @@
         <v>46202</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="123" t="s">
+      <c r="D3" s="109" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
+      <c r="E3" s="109"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="109"/>
+      <c r="H3" s="109"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -3368,12 +3388,12 @@
       <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="125" t="s">
+      <c r="E4" s="110" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="126"/>
-      <c r="G4" s="126"/>
-      <c r="H4" s="127"/>
+      <c r="F4" s="111"/>
+      <c r="G4" s="111"/>
+      <c r="H4" s="112"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -3447,12 +3467,12 @@
       <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="117" t="s">
+      <c r="E5" s="113" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="118"/>
-      <c r="G5" s="118"/>
-      <c r="H5" s="119"/>
+      <c r="F5" s="114"/>
+      <c r="G5" s="114"/>
+      <c r="H5" s="115"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -3526,12 +3546,12 @@
       <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="117" t="s">
+      <c r="E6" s="113" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="118"/>
-      <c r="G6" s="118"/>
-      <c r="H6" s="119"/>
+      <c r="F6" s="114"/>
+      <c r="G6" s="114"/>
+      <c r="H6" s="115"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -3605,12 +3625,12 @@
       <c r="D7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="117" t="s">
+      <c r="E7" s="113" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="118"/>
-      <c r="G7" s="118"/>
-      <c r="H7" s="119"/>
+      <c r="F7" s="114"/>
+      <c r="G7" s="114"/>
+      <c r="H7" s="115"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -3684,12 +3704,12 @@
       <c r="D8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="117" t="s">
+      <c r="E8" s="113" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="118"/>
-      <c r="G8" s="118"/>
-      <c r="H8" s="119"/>
+      <c r="F8" s="114"/>
+      <c r="G8" s="114"/>
+      <c r="H8" s="115"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -3763,12 +3783,12 @@
       <c r="D9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="117" t="s">
+      <c r="E9" s="113" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="118"/>
-      <c r="G9" s="118"/>
-      <c r="H9" s="119"/>
+      <c r="F9" s="114"/>
+      <c r="G9" s="114"/>
+      <c r="H9" s="115"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -3842,12 +3862,12 @@
       <c r="D10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="120" t="s">
+      <c r="E10" s="125" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="121"/>
-      <c r="G10" s="121"/>
-      <c r="H10" s="122"/>
+      <c r="F10" s="126"/>
+      <c r="G10" s="126"/>
+      <c r="H10" s="127"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -4128,16 +4148,16 @@
       <c r="BQ13" s="1"/>
     </row>
     <row r="14" spans="1:69" ht="15">
-      <c r="A14" s="123" t="s">
+      <c r="A14" s="109" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="123"/>
-      <c r="C14" s="123"/>
-      <c r="D14" s="123"/>
-      <c r="E14" s="123"/>
-      <c r="F14" s="123"/>
-      <c r="G14" s="123"/>
-      <c r="H14" s="123"/>
+      <c r="B14" s="109"/>
+      <c r="C14" s="109"/>
+      <c r="D14" s="109"/>
+      <c r="E14" s="109"/>
+      <c r="F14" s="109"/>
+      <c r="G14" s="109"/>
+      <c r="H14" s="109"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -4201,16 +4221,16 @@
       <c r="BQ14" s="1"/>
     </row>
     <row r="15" spans="1:69" ht="15">
-      <c r="A15" s="108" t="s">
+      <c r="A15" s="116" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="109"/>
-      <c r="C15" s="109"/>
-      <c r="D15" s="109"/>
-      <c r="E15" s="109"/>
-      <c r="F15" s="109"/>
-      <c r="G15" s="109"/>
-      <c r="H15" s="110"/>
+      <c r="B15" s="117"/>
+      <c r="C15" s="117"/>
+      <c r="D15" s="117"/>
+      <c r="E15" s="117"/>
+      <c r="F15" s="117"/>
+      <c r="G15" s="117"/>
+      <c r="H15" s="118"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -4274,14 +4294,14 @@
       <c r="BQ15" s="1"/>
     </row>
     <row r="16" spans="1:69" ht="15">
-      <c r="A16" s="111"/>
-      <c r="B16" s="112"/>
-      <c r="C16" s="112"/>
-      <c r="D16" s="112"/>
-      <c r="E16" s="112"/>
-      <c r="F16" s="112"/>
-      <c r="G16" s="112"/>
-      <c r="H16" s="113"/>
+      <c r="A16" s="119"/>
+      <c r="B16" s="120"/>
+      <c r="C16" s="120"/>
+      <c r="D16" s="120"/>
+      <c r="E16" s="120"/>
+      <c r="F16" s="120"/>
+      <c r="G16" s="120"/>
+      <c r="H16" s="121"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -4345,14 +4365,14 @@
       <c r="BQ16" s="1"/>
     </row>
     <row r="17" spans="1:69" ht="15">
-      <c r="A17" s="111"/>
-      <c r="B17" s="112"/>
-      <c r="C17" s="112"/>
-      <c r="D17" s="112"/>
-      <c r="E17" s="112"/>
-      <c r="F17" s="112"/>
-      <c r="G17" s="112"/>
-      <c r="H17" s="113"/>
+      <c r="A17" s="119"/>
+      <c r="B17" s="120"/>
+      <c r="C17" s="120"/>
+      <c r="D17" s="120"/>
+      <c r="E17" s="120"/>
+      <c r="F17" s="120"/>
+      <c r="G17" s="120"/>
+      <c r="H17" s="121"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -4416,14 +4436,14 @@
       <c r="BQ17" s="1"/>
     </row>
     <row r="18" spans="1:69" ht="15">
-      <c r="A18" s="114"/>
-      <c r="B18" s="115"/>
-      <c r="C18" s="115"/>
-      <c r="D18" s="115"/>
-      <c r="E18" s="115"/>
-      <c r="F18" s="115"/>
-      <c r="G18" s="115"/>
-      <c r="H18" s="116"/>
+      <c r="A18" s="122"/>
+      <c r="B18" s="123"/>
+      <c r="C18" s="123"/>
+      <c r="D18" s="123"/>
+      <c r="E18" s="123"/>
+      <c r="F18" s="123"/>
+      <c r="G18" s="123"/>
+      <c r="H18" s="124"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -10310,17 +10330,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:H6"/>
     <mergeCell ref="A15:H18"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="E9:H9"/>
     <mergeCell ref="E10:H10"/>
     <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10341,28 +10361,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
-      <c r="I1" s="124"/>
-      <c r="J1" s="124"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="124"/>
-      <c r="M1" s="124"/>
-      <c r="N1" s="124"/>
-      <c r="O1" s="124"/>
-      <c r="P1" s="124"/>
-      <c r="Q1" s="124"/>
-      <c r="R1" s="124"/>
-      <c r="S1" s="124"/>
-      <c r="T1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="108"/>
+      <c r="M1" s="108"/>
+      <c r="N1" s="108"/>
+      <c r="O1" s="108"/>
+      <c r="P1" s="108"/>
+      <c r="Q1" s="108"/>
+      <c r="R1" s="108"/>
+      <c r="S1" s="108"/>
+      <c r="T1" s="108"/>
       <c r="U1" s="107"/>
       <c r="V1" s="107"/>
       <c r="W1" s="107"/>
@@ -17703,35 +17723,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="15">
-      <c r="A1" s="123" t="s">
+      <c r="A1" s="109" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="123"/>
+      <c r="B1" s="109"/>
       <c r="C1" s="45">
         <v>46202</v>
       </c>
-      <c r="D1" s="123" t="s">
+      <c r="D1" s="109" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="123"/>
-      <c r="F1" s="123"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
       <c r="G1" s="4">
         <v>576</v>
       </c>
-      <c r="H1" s="123" t="s">
+      <c r="H1" s="109" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="123"/>
-      <c r="J1" s="123"/>
-      <c r="K1" s="123"/>
-      <c r="L1" s="123" t="s">
+      <c r="I1" s="109"/>
+      <c r="J1" s="109"/>
+      <c r="K1" s="109"/>
+      <c r="L1" s="109" t="s">
         <v>83</v>
       </c>
-      <c r="M1" s="123"/>
-      <c r="N1" s="123"/>
-      <c r="O1" s="123"/>
-      <c r="P1" s="123"/>
-      <c r="Q1" s="123"/>
+      <c r="M1" s="109"/>
+      <c r="N1" s="109"/>
+      <c r="O1" s="109"/>
+      <c r="P1" s="109"/>
+      <c r="Q1" s="109"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -18353,24 +18373,24 @@
         <v>46208</v>
       </c>
       <c r="L6" s="47" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
       <c r="M6" s="49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N6" s="47">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="O6" s="47">
         <f t="shared" ref="O6:O37" si="3">IF(N6="","",N6-F6)</f>
-        <v>-1.5</v>
+        <v>-2.5</v>
       </c>
       <c r="P6" s="47">
         <f t="shared" ref="P6:P37" si="4">MAX(F6*(1-M6),0)</f>
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="R6" s="50" t="s">
         <v>57</v>
@@ -18429,16 +18449,16 @@
     </row>
     <row r="7" spans="1:69" ht="42" customHeight="1">
       <c r="A7" s="20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="22" t="s">
+        <v>158</v>
+      </c>
+      <c r="D7" s="22" t="s">
         <v>159</v>
-      </c>
-      <c r="D7" s="22" t="s">
-        <v>160</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>153</v>
@@ -18468,7 +18488,7 @@
         <v>422</v>
       </c>
       <c r="M7" s="49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="47"/>
       <c r="O7" s="47" t="str">
@@ -18477,9 +18497,11 @@
       </c>
       <c r="P7" s="47">
         <f t="shared" si="4"/>
-        <v>4</v>
-      </c>
-      <c r="Q7" s="25"/>
+        <v>0</v>
+      </c>
+      <c r="Q7" s="25" t="s">
+        <v>424</v>
+      </c>
       <c r="R7" s="50" t="s">
         <v>57</v>
       </c>
@@ -18537,16 +18559,16 @@
     </row>
     <row r="8" spans="1:69" ht="42" customHeight="1">
       <c r="A8" s="20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C8" s="22" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="22" t="s">
         <v>162</v>
-      </c>
-      <c r="D8" s="22" t="s">
-        <v>163</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>153</v>
@@ -18573,10 +18595,10 @@
         <v>46215</v>
       </c>
       <c r="L8" s="47" t="s">
-        <v>157</v>
+        <v>425</v>
       </c>
       <c r="M8" s="49">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="N8" s="47"/>
       <c r="O8" s="47" t="str">
@@ -18585,9 +18607,11 @@
       </c>
       <c r="P8" s="47">
         <f t="shared" si="4"/>
-        <v>4</v>
-      </c>
-      <c r="Q8" s="25"/>
+        <v>2</v>
+      </c>
+      <c r="Q8" s="25" t="s">
+        <v>426</v>
+      </c>
       <c r="R8" s="55" t="s">
         <v>57</v>
       </c>
@@ -18647,19 +18671,19 @@
     </row>
     <row r="9" spans="1:69" ht="42" customHeight="1">
       <c r="A9" s="20" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C9" s="22" t="s">
+        <v>164</v>
+      </c>
+      <c r="D9" s="22" t="s">
         <v>165</v>
       </c>
-      <c r="D9" s="22" t="s">
-        <v>166</v>
-      </c>
       <c r="E9" s="22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F9" s="47">
         <v>4</v>
@@ -18683,7 +18707,7 @@
         <v>46215</v>
       </c>
       <c r="L9" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M9" s="49">
         <v>0</v>
@@ -18767,7 +18791,7 @@
         <v>169</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F10" s="47">
         <v>12</v>
@@ -18791,10 +18815,10 @@
         <v>46565</v>
       </c>
       <c r="L10" s="47" t="s">
-        <v>157</v>
+        <v>425</v>
       </c>
       <c r="M10" s="49">
-        <v>0</v>
+        <v>0.02</v>
       </c>
       <c r="N10" s="47"/>
       <c r="O10" s="47" t="str">
@@ -18803,9 +18827,11 @@
       </c>
       <c r="P10" s="47">
         <f t="shared" si="4"/>
-        <v>12</v>
-      </c>
-      <c r="Q10" s="25"/>
+        <v>11.76</v>
+      </c>
+      <c r="Q10" s="25" t="s">
+        <v>427</v>
+      </c>
       <c r="R10" s="55" t="s">
         <v>57</v>
       </c>
@@ -18977,7 +19003,7 @@
         <v>172</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F11" s="47">
         <v>6</v>
@@ -19001,7 +19027,7 @@
         <v>46565</v>
       </c>
       <c r="L11" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M11" s="49">
         <v>0</v>
@@ -19181,7 +19207,7 @@
         <v>175</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F12" s="47">
         <v>6</v>
@@ -19205,7 +19231,7 @@
         <v>46565</v>
       </c>
       <c r="L12" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M12" s="49">
         <v>0</v>
@@ -19375,7 +19401,7 @@
         <v>178</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F13" s="47">
         <v>8</v>
@@ -19399,7 +19425,7 @@
         <v>46222</v>
       </c>
       <c r="L13" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M13" s="49">
         <v>0</v>
@@ -19507,7 +19533,7 @@
         <v>46229</v>
       </c>
       <c r="L14" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M14" s="49">
         <v>0</v>
@@ -19617,7 +19643,7 @@
         <v>46236</v>
       </c>
       <c r="L15" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M15" s="49">
         <v>0</v>
@@ -19727,7 +19753,7 @@
         <v>46250</v>
       </c>
       <c r="L16" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M16" s="49">
         <v>0</v>
@@ -19839,7 +19865,7 @@
         <v>46257</v>
       </c>
       <c r="L17" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M17" s="49">
         <v>0</v>
@@ -19949,7 +19975,7 @@
         <v>46257</v>
       </c>
       <c r="L18" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M18" s="49">
         <v>0</v>
@@ -20057,7 +20083,7 @@
         <v>46264</v>
       </c>
       <c r="L19" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M19" s="49">
         <v>0</v>
@@ -20165,10 +20191,10 @@
         <v>46271</v>
       </c>
       <c r="L20" s="47" t="s">
-        <v>157</v>
+        <v>425</v>
       </c>
       <c r="M20" s="49">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="N20" s="47"/>
       <c r="O20" s="47" t="str">
@@ -20177,9 +20203,11 @@
       </c>
       <c r="P20" s="47">
         <f t="shared" si="4"/>
-        <v>10</v>
-      </c>
-      <c r="Q20" s="25"/>
+        <v>8</v>
+      </c>
+      <c r="Q20" s="25" t="s">
+        <v>428</v>
+      </c>
       <c r="R20" s="57"/>
       <c r="S20" s="53"/>
       <c r="T20" s="53"/>
@@ -20273,7 +20301,7 @@
         <v>46278</v>
       </c>
       <c r="L21" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M21" s="49">
         <v>0</v>
@@ -20383,10 +20411,10 @@
         <v>46285</v>
       </c>
       <c r="L22" s="47" t="s">
-        <v>157</v>
+        <v>422</v>
       </c>
       <c r="M22" s="49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N22" s="47"/>
       <c r="O22" s="47" t="str">
@@ -20395,9 +20423,11 @@
       </c>
       <c r="P22" s="47">
         <f t="shared" si="4"/>
-        <v>14</v>
-      </c>
-      <c r="Q22" s="25"/>
+        <v>0</v>
+      </c>
+      <c r="Q22" s="25" t="s">
+        <v>429</v>
+      </c>
       <c r="R22" s="57"/>
       <c r="S22" s="53"/>
       <c r="T22" s="53"/>
@@ -20493,7 +20523,7 @@
         <v>46292</v>
       </c>
       <c r="L23" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M23" s="49">
         <v>0</v>
@@ -20603,7 +20633,7 @@
         <v>46299</v>
       </c>
       <c r="L24" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M24" s="49">
         <v>0</v>
@@ -20713,7 +20743,7 @@
         <v>46306</v>
       </c>
       <c r="L25" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M25" s="49">
         <v>0</v>
@@ -20823,7 +20853,7 @@
         <v>46306</v>
       </c>
       <c r="L26" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M26" s="49">
         <v>0</v>
@@ -20931,7 +20961,7 @@
         <v>46313</v>
       </c>
       <c r="L27" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M27" s="49">
         <v>0</v>
@@ -21039,7 +21069,7 @@
         <v>46327</v>
       </c>
       <c r="L28" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M28" s="49">
         <v>0</v>
@@ -21149,7 +21179,7 @@
         <v>46334</v>
       </c>
       <c r="L29" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M29" s="49">
         <v>0</v>
@@ -21259,7 +21289,7 @@
         <v>46341</v>
       </c>
       <c r="L30" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M30" s="49">
         <v>0</v>
@@ -21369,7 +21399,7 @@
         <v>46341</v>
       </c>
       <c r="L31" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M31" s="49">
         <v>0</v>
@@ -21477,7 +21507,7 @@
         <v>46348</v>
       </c>
       <c r="L32" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M32" s="49">
         <v>0</v>
@@ -21585,7 +21615,7 @@
         <v>46355</v>
       </c>
       <c r="L33" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M33" s="49">
         <v>0</v>
@@ -21695,7 +21725,7 @@
         <v>46362</v>
       </c>
       <c r="L34" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M34" s="49">
         <v>0</v>
@@ -21805,7 +21835,7 @@
         <v>46369</v>
       </c>
       <c r="L35" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M35" s="49">
         <v>0</v>
@@ -21913,7 +21943,7 @@
         <v>46376</v>
       </c>
       <c r="L36" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M36" s="49">
         <v>0</v>
@@ -22021,7 +22051,7 @@
         <v>46383</v>
       </c>
       <c r="L37" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M37" s="49">
         <v>0</v>
@@ -22131,7 +22161,7 @@
         <v>46397</v>
       </c>
       <c r="L38" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M38" s="49">
         <v>0</v>
@@ -22243,7 +22273,7 @@
         <v>46404</v>
       </c>
       <c r="L39" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M39" s="49">
         <v>0</v>
@@ -22353,7 +22383,7 @@
         <v>46411</v>
       </c>
       <c r="L40" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M40" s="49">
         <v>0</v>
@@ -22463,7 +22493,7 @@
         <v>46418</v>
       </c>
       <c r="L41" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M41" s="49">
         <v>0</v>
@@ -22573,7 +22603,7 @@
         <v>46425</v>
       </c>
       <c r="L42" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M42" s="49">
         <v>0</v>
@@ -22681,7 +22711,7 @@
         <v>46432</v>
       </c>
       <c r="L43" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M43" s="49">
         <v>0</v>
@@ -22789,7 +22819,7 @@
         <v>46446</v>
       </c>
       <c r="L44" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M44" s="49">
         <v>0</v>
@@ -22899,7 +22929,7 @@
         <v>46453</v>
       </c>
       <c r="L45" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M45" s="49">
         <v>0</v>
@@ -23009,7 +23039,7 @@
         <v>46453</v>
       </c>
       <c r="L46" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M46" s="49">
         <v>0</v>
@@ -23117,7 +23147,7 @@
         <v>46467</v>
       </c>
       <c r="L47" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M47" s="49">
         <v>0</v>
@@ -23227,7 +23257,7 @@
         <v>46474</v>
       </c>
       <c r="L48" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M48" s="49">
         <v>0</v>
@@ -23337,7 +23367,7 @@
         <v>46488</v>
       </c>
       <c r="L49" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M49" s="49">
         <v>0</v>
@@ -23447,7 +23477,7 @@
         <v>46495</v>
       </c>
       <c r="L50" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M50" s="49">
         <v>0</v>
@@ -23555,7 +23585,7 @@
         <v>46502</v>
       </c>
       <c r="L51" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M51" s="49">
         <v>0</v>
@@ -23663,7 +23693,7 @@
         <v>46509</v>
       </c>
       <c r="L52" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M52" s="49">
         <v>0</v>
@@ -23773,7 +23803,7 @@
         <v>46516</v>
       </c>
       <c r="L53" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M53" s="49">
         <v>0</v>
@@ -23883,7 +23913,7 @@
         <v>46523</v>
       </c>
       <c r="L54" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M54" s="49">
         <v>0</v>
@@ -23993,7 +24023,7 @@
         <v>46530</v>
       </c>
       <c r="L55" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M55" s="49">
         <v>0</v>
@@ -24103,7 +24133,7 @@
         <v>46530</v>
       </c>
       <c r="L56" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M56" s="49">
         <v>0</v>
@@ -24211,7 +24241,7 @@
         <v>46537</v>
       </c>
       <c r="L57" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M57" s="49">
         <v>0</v>
@@ -24319,7 +24349,7 @@
         <v>46544</v>
       </c>
       <c r="L58" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M58" s="49">
         <v>0</v>
@@ -24429,7 +24459,7 @@
         <v>46551</v>
       </c>
       <c r="L59" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M59" s="49">
         <v>0</v>
@@ -24539,7 +24569,7 @@
         <v>46551</v>
       </c>
       <c r="L60" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M60" s="49">
         <v>0</v>
@@ -24647,7 +24677,7 @@
         <v>46558</v>
       </c>
       <c r="L61" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M61" s="49">
         <v>0</v>
@@ -24755,7 +24785,7 @@
         <v>46565</v>
       </c>
       <c r="L62" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M62" s="49">
         <v>0</v>
@@ -24865,7 +24895,7 @@
         <v>46565</v>
       </c>
       <c r="L63" s="47" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="M63" s="49">
         <v>0</v>
@@ -27596,6 +27626,13 @@
         <cfvo type="max"/>
         <color rgb="FF2563EB"/>
       </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF2563EB"/>
+      </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{B05FFF90-18D4-A5A7-8560-2BA14D3F5BBD}</x14:id>
@@ -27654,20 +27691,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>329</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
-      <c r="I1" s="124"/>
-      <c r="J1" s="124"/>
-      <c r="K1" s="124"/>
-      <c r="L1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
+      <c r="I1" s="108"/>
+      <c r="J1" s="108"/>
+      <c r="K1" s="108"/>
+      <c r="L1" s="108"/>
       <c r="M1" s="107"/>
       <c r="N1" s="107"/>
       <c r="O1" s="107"/>
@@ -27892,7 +27929,7 @@
       <c r="BP3" s="1"/>
       <c r="BQ3" s="1"/>
     </row>
-    <row r="4" spans="1:69" ht="15">
+    <row r="4" spans="1:69" ht="81">
       <c r="A4" s="84">
         <v>1</v>
       </c>
@@ -27905,10 +27942,12 @@
       <c r="D4" s="86">
         <v>11</v>
       </c>
-      <c r="E4" s="86"/>
-      <c r="F4" s="86" t="str">
+      <c r="E4" s="86">
+        <v>1.5</v>
+      </c>
+      <c r="F4" s="86">
         <f t="shared" ref="F4:F35" si="0">IF(E4="","",E4-D4)</f>
-        <v/>
+        <v>-9.5</v>
       </c>
       <c r="G4" s="86">
         <f>D4</f>
@@ -27916,7 +27955,7 @@
       </c>
       <c r="H4" s="86">
         <f>IF(E4="",0,E4)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I4" s="86">
         <f t="shared" ref="I4:I35" si="1">MAX(576-G4,0)</f>
@@ -27926,9 +27965,11 @@
         <v>339</v>
       </c>
       <c r="K4" s="86" t="s">
-        <v>422</v>
-      </c>
-      <c r="L4" s="87"/>
+        <v>425</v>
+      </c>
+      <c r="L4" s="87" t="s">
+        <v>430</v>
+      </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
       <c r="O4" s="1"/>
@@ -28011,7 +28052,7 @@
       </c>
       <c r="H5" s="86">
         <f t="shared" ref="H5:H36" si="3">H4+IF(E5="",0,E5)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I5" s="86">
         <f t="shared" si="1"/>
@@ -28021,7 +28062,7 @@
         <v>339</v>
       </c>
       <c r="K5" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L5" s="87"/>
       <c r="M5" s="1"/>
@@ -28106,7 +28147,7 @@
       </c>
       <c r="H6" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I6" s="86">
         <f t="shared" si="1"/>
@@ -28116,7 +28157,7 @@
         <v>340</v>
       </c>
       <c r="K6" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L6" s="87"/>
       <c r="M6" s="1"/>
@@ -28201,7 +28242,7 @@
       </c>
       <c r="H7" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I7" s="86">
         <f t="shared" si="1"/>
@@ -28211,7 +28252,7 @@
         <v>340</v>
       </c>
       <c r="K7" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L7" s="87"/>
       <c r="M7" s="1"/>
@@ -28296,7 +28337,7 @@
       </c>
       <c r="H8" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I8" s="86">
         <f t="shared" si="1"/>
@@ -28306,7 +28347,7 @@
         <v>340</v>
       </c>
       <c r="K8" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L8" s="87"/>
       <c r="M8" s="1"/>
@@ -28391,7 +28432,7 @@
       </c>
       <c r="H9" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I9" s="86">
         <f t="shared" si="1"/>
@@ -28401,7 +28442,7 @@
         <v>340</v>
       </c>
       <c r="K9" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L9" s="87"/>
       <c r="M9" s="1"/>
@@ -28486,7 +28527,7 @@
       </c>
       <c r="H10" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I10" s="86">
         <f t="shared" si="1"/>
@@ -28496,7 +28537,7 @@
         <v>340</v>
       </c>
       <c r="K10" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L10" s="87"/>
       <c r="M10" s="1"/>
@@ -28581,7 +28622,7 @@
       </c>
       <c r="H11" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I11" s="86">
         <f t="shared" si="1"/>
@@ -28591,7 +28632,7 @@
         <v>340</v>
       </c>
       <c r="K11" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L11" s="87"/>
       <c r="M11" s="1"/>
@@ -28676,7 +28717,7 @@
       </c>
       <c r="H12" s="90">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I12" s="90">
         <f t="shared" si="1"/>
@@ -28686,7 +28727,7 @@
         <v>340</v>
       </c>
       <c r="K12" s="90" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L12" s="91"/>
       <c r="M12" s="1"/>
@@ -28771,7 +28812,7 @@
       </c>
       <c r="H13" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I13" s="86">
         <f t="shared" si="1"/>
@@ -28781,7 +28822,7 @@
         <v>341</v>
       </c>
       <c r="K13" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L13" s="87"/>
       <c r="M13" s="1"/>
@@ -28866,7 +28907,7 @@
       </c>
       <c r="H14" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I14" s="86">
         <f t="shared" si="1"/>
@@ -28876,7 +28917,7 @@
         <v>341</v>
       </c>
       <c r="K14" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L14" s="87"/>
       <c r="M14" s="1"/>
@@ -28961,7 +29002,7 @@
       </c>
       <c r="H15" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I15" s="86">
         <f t="shared" si="1"/>
@@ -28971,7 +29012,7 @@
         <v>341</v>
       </c>
       <c r="K15" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L15" s="87"/>
       <c r="M15" s="1"/>
@@ -29056,7 +29097,7 @@
       </c>
       <c r="H16" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I16" s="86">
         <f t="shared" si="1"/>
@@ -29066,7 +29107,7 @@
         <v>341</v>
       </c>
       <c r="K16" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L16" s="87"/>
       <c r="M16" s="1"/>
@@ -29151,7 +29192,7 @@
       </c>
       <c r="H17" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I17" s="86">
         <f t="shared" si="1"/>
@@ -29161,7 +29202,7 @@
         <v>341</v>
       </c>
       <c r="K17" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L17" s="87"/>
       <c r="M17" s="1"/>
@@ -29246,7 +29287,7 @@
       </c>
       <c r="H18" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I18" s="86">
         <f t="shared" si="1"/>
@@ -29256,7 +29297,7 @@
         <v>341</v>
       </c>
       <c r="K18" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L18" s="87"/>
       <c r="M18" s="1"/>
@@ -29341,7 +29382,7 @@
       </c>
       <c r="H19" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I19" s="86">
         <f t="shared" si="1"/>
@@ -29351,7 +29392,7 @@
         <v>341</v>
       </c>
       <c r="K19" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L19" s="87"/>
       <c r="M19" s="1"/>
@@ -29436,7 +29477,7 @@
       </c>
       <c r="H20" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I20" s="86">
         <f t="shared" si="1"/>
@@ -29446,7 +29487,7 @@
         <v>342</v>
       </c>
       <c r="K20" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L20" s="87"/>
       <c r="M20" s="1"/>
@@ -29531,7 +29572,7 @@
       </c>
       <c r="H21" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I21" s="86">
         <f t="shared" si="1"/>
@@ -29541,7 +29582,7 @@
         <v>342</v>
       </c>
       <c r="K21" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L21" s="87"/>
       <c r="M21" s="1"/>
@@ -29626,7 +29667,7 @@
       </c>
       <c r="H22" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I22" s="86">
         <f t="shared" si="1"/>
@@ -29636,7 +29677,7 @@
         <v>342</v>
       </c>
       <c r="K22" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L22" s="87"/>
       <c r="M22" s="1"/>
@@ -29721,7 +29762,7 @@
       </c>
       <c r="H23" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I23" s="86">
         <f t="shared" si="1"/>
@@ -29731,7 +29772,7 @@
         <v>342</v>
       </c>
       <c r="K23" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L23" s="87"/>
       <c r="M23" s="1"/>
@@ -29816,7 +29857,7 @@
       </c>
       <c r="H24" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I24" s="86">
         <f t="shared" si="1"/>
@@ -29826,7 +29867,7 @@
         <v>342</v>
       </c>
       <c r="K24" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L24" s="87"/>
       <c r="M24" s="1"/>
@@ -29911,7 +29952,7 @@
       </c>
       <c r="H25" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I25" s="86">
         <f t="shared" si="1"/>
@@ -29921,7 +29962,7 @@
         <v>342</v>
       </c>
       <c r="K25" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L25" s="87"/>
       <c r="M25" s="1"/>
@@ -30006,7 +30047,7 @@
       </c>
       <c r="H26" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I26" s="86">
         <f t="shared" si="1"/>
@@ -30016,7 +30057,7 @@
         <v>342</v>
       </c>
       <c r="K26" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L26" s="87"/>
       <c r="M26" s="1"/>
@@ -30101,7 +30142,7 @@
       </c>
       <c r="H27" s="90">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I27" s="90">
         <f t="shared" si="1"/>
@@ -30111,7 +30152,7 @@
         <v>342</v>
       </c>
       <c r="K27" s="90" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L27" s="91"/>
       <c r="M27" s="1"/>
@@ -30196,7 +30237,7 @@
       </c>
       <c r="H28" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I28" s="86">
         <f t="shared" si="1"/>
@@ -30206,7 +30247,7 @@
         <v>343</v>
       </c>
       <c r="K28" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L28" s="87"/>
       <c r="M28" s="1"/>
@@ -30291,7 +30332,7 @@
       </c>
       <c r="H29" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I29" s="86">
         <f t="shared" si="1"/>
@@ -30301,7 +30342,7 @@
         <v>343</v>
       </c>
       <c r="K29" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L29" s="87"/>
       <c r="M29" s="1"/>
@@ -30386,7 +30427,7 @@
       </c>
       <c r="H30" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I30" s="86">
         <f t="shared" si="1"/>
@@ -30396,7 +30437,7 @@
         <v>343</v>
       </c>
       <c r="K30" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L30" s="87"/>
       <c r="M30" s="1"/>
@@ -30481,7 +30522,7 @@
       </c>
       <c r="H31" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I31" s="86">
         <f t="shared" si="1"/>
@@ -30491,7 +30532,7 @@
         <v>343</v>
       </c>
       <c r="K31" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L31" s="87"/>
       <c r="M31" s="1"/>
@@ -30576,7 +30617,7 @@
       </c>
       <c r="H32" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I32" s="86">
         <f t="shared" si="1"/>
@@ -30586,7 +30627,7 @@
         <v>343</v>
       </c>
       <c r="K32" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L32" s="87"/>
       <c r="M32" s="1"/>
@@ -30671,7 +30712,7 @@
       </c>
       <c r="H33" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I33" s="86">
         <f t="shared" si="1"/>
@@ -30681,7 +30722,7 @@
         <v>343</v>
       </c>
       <c r="K33" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L33" s="87"/>
       <c r="M33" s="1"/>
@@ -30766,7 +30807,7 @@
       </c>
       <c r="H34" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I34" s="86">
         <f t="shared" si="1"/>
@@ -30776,7 +30817,7 @@
         <v>343</v>
       </c>
       <c r="K34" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L34" s="87"/>
       <c r="M34" s="1"/>
@@ -30861,7 +30902,7 @@
       </c>
       <c r="H35" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I35" s="86">
         <f t="shared" si="1"/>
@@ -30871,7 +30912,7 @@
         <v>343</v>
       </c>
       <c r="K35" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L35" s="87"/>
       <c r="M35" s="1"/>
@@ -30956,7 +30997,7 @@
       </c>
       <c r="H36" s="86">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I36" s="86">
         <f t="shared" ref="I36:I55" si="5">MAX(576-G36,0)</f>
@@ -30966,7 +31007,7 @@
         <v>344</v>
       </c>
       <c r="K36" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L36" s="87"/>
       <c r="M36" s="1"/>
@@ -31051,7 +31092,7 @@
       </c>
       <c r="H37" s="86">
         <f t="shared" ref="H37:H55" si="7">H36+IF(E37="",0,E37)</f>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I37" s="86">
         <f t="shared" si="5"/>
@@ -31061,7 +31102,7 @@
         <v>344</v>
       </c>
       <c r="K37" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L37" s="87"/>
       <c r="M37" s="1"/>
@@ -31146,7 +31187,7 @@
       </c>
       <c r="H38" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I38" s="86">
         <f t="shared" si="5"/>
@@ -31156,7 +31197,7 @@
         <v>344</v>
       </c>
       <c r="K38" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L38" s="87"/>
       <c r="M38" s="1"/>
@@ -31241,7 +31282,7 @@
       </c>
       <c r="H39" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I39" s="86">
         <f t="shared" si="5"/>
@@ -31251,7 +31292,7 @@
         <v>344</v>
       </c>
       <c r="K39" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L39" s="87"/>
       <c r="M39" s="1"/>
@@ -31336,7 +31377,7 @@
       </c>
       <c r="H40" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I40" s="86">
         <f t="shared" si="5"/>
@@ -31346,7 +31387,7 @@
         <v>344</v>
       </c>
       <c r="K40" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L40" s="87"/>
       <c r="M40" s="1"/>
@@ -31431,7 +31472,7 @@
       </c>
       <c r="H41" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I41" s="86">
         <f t="shared" si="5"/>
@@ -31441,7 +31482,7 @@
         <v>344</v>
       </c>
       <c r="K41" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L41" s="87"/>
       <c r="M41" s="1"/>
@@ -31526,7 +31567,7 @@
       </c>
       <c r="H42" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I42" s="86">
         <f t="shared" si="5"/>
@@ -31536,7 +31577,7 @@
         <v>344</v>
       </c>
       <c r="K42" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L42" s="87"/>
       <c r="M42" s="1"/>
@@ -31621,7 +31662,7 @@
       </c>
       <c r="H43" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I43" s="86">
         <f t="shared" si="5"/>
@@ -31631,7 +31672,7 @@
         <v>344</v>
       </c>
       <c r="K43" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L43" s="87"/>
       <c r="M43" s="1"/>
@@ -31716,7 +31757,7 @@
       </c>
       <c r="H44" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I44" s="86">
         <f t="shared" si="5"/>
@@ -31726,7 +31767,7 @@
         <v>344</v>
       </c>
       <c r="K44" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L44" s="87"/>
       <c r="M44" s="1"/>
@@ -31811,7 +31852,7 @@
       </c>
       <c r="H45" s="90">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I45" s="90">
         <f t="shared" si="5"/>
@@ -31821,7 +31862,7 @@
         <v>344</v>
       </c>
       <c r="K45" s="90" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L45" s="91"/>
       <c r="M45" s="1"/>
@@ -31906,7 +31947,7 @@
       </c>
       <c r="H46" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I46" s="86">
         <f t="shared" si="5"/>
@@ -31916,7 +31957,7 @@
         <v>345</v>
       </c>
       <c r="K46" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L46" s="87"/>
       <c r="M46" s="1"/>
@@ -32001,7 +32042,7 @@
       </c>
       <c r="H47" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I47" s="86">
         <f t="shared" si="5"/>
@@ -32011,7 +32052,7 @@
         <v>345</v>
       </c>
       <c r="K47" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L47" s="87"/>
       <c r="M47" s="1"/>
@@ -32096,7 +32137,7 @@
       </c>
       <c r="H48" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I48" s="86">
         <f t="shared" si="5"/>
@@ -32106,7 +32147,7 @@
         <v>345</v>
       </c>
       <c r="K48" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L48" s="87"/>
       <c r="M48" s="1"/>
@@ -32191,7 +32232,7 @@
       </c>
       <c r="H49" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I49" s="86">
         <f t="shared" si="5"/>
@@ -32201,7 +32242,7 @@
         <v>345</v>
       </c>
       <c r="K49" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L49" s="87"/>
       <c r="M49" s="1"/>
@@ -32286,7 +32327,7 @@
       </c>
       <c r="H50" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I50" s="86">
         <f t="shared" si="5"/>
@@ -32296,7 +32337,7 @@
         <v>345</v>
       </c>
       <c r="K50" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L50" s="87"/>
       <c r="M50" s="1"/>
@@ -32381,7 +32422,7 @@
       </c>
       <c r="H51" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I51" s="86">
         <f t="shared" si="5"/>
@@ -32391,7 +32432,7 @@
         <v>346</v>
       </c>
       <c r="K51" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L51" s="87"/>
       <c r="M51" s="1"/>
@@ -32476,7 +32517,7 @@
       </c>
       <c r="H52" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I52" s="86">
         <f t="shared" si="5"/>
@@ -32486,7 +32527,7 @@
         <v>346</v>
       </c>
       <c r="K52" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L52" s="87"/>
       <c r="M52" s="1"/>
@@ -32571,7 +32612,7 @@
       </c>
       <c r="H53" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I53" s="86">
         <f t="shared" si="5"/>
@@ -32581,7 +32622,7 @@
         <v>346</v>
       </c>
       <c r="K53" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L53" s="87"/>
       <c r="M53" s="1"/>
@@ -32666,7 +32707,7 @@
       </c>
       <c r="H54" s="86">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I54" s="86">
         <f t="shared" si="5"/>
@@ -32676,7 +32717,7 @@
         <v>346</v>
       </c>
       <c r="K54" s="86" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L54" s="87"/>
       <c r="M54" s="1"/>
@@ -32761,7 +32802,7 @@
       </c>
       <c r="H55" s="90">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>1.5</v>
       </c>
       <c r="I55" s="90">
         <f t="shared" si="5"/>
@@ -32771,7 +32812,7 @@
         <v>346</v>
       </c>
       <c r="K55" s="90" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="L55" s="91"/>
       <c r="M55" s="1"/>
@@ -36045,6 +36086,13 @@
         <cfvo type="max"/>
         <color rgb="FF2563EB"/>
       </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="7">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF2563EB"/>
+      </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{B9CF9B83-EEEF-806F-3865-A7F6C560F42A}</x14:id>
@@ -36061,6 +36109,13 @@
       </dataBar>
     </cfRule>
     <cfRule type="dataBar" priority="6">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF16A34A"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="8">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -36134,16 +36189,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>347</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -43370,16 +43425,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>350</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
-      <c r="E1" s="124"/>
-      <c r="F1" s="124"/>
-      <c r="G1" s="124"/>
-      <c r="H1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="108"/>
+      <c r="F1" s="108"/>
+      <c r="G1" s="108"/>
+      <c r="H1" s="108"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -43514,16 +43569,16 @@
       <c r="BQ2" s="1"/>
     </row>
     <row r="3" spans="1:69" ht="15">
-      <c r="A3" s="123" t="s">
+      <c r="A3" s="109" t="s">
         <v>351</v>
       </c>
-      <c r="B3" s="123"/>
-      <c r="C3" s="123"/>
-      <c r="D3" s="123"/>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="109"/>
+      <c r="F3" s="109"/>
+      <c r="G3" s="109"/>
+      <c r="H3" s="109"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -45271,16 +45326,16 @@
       <c r="BQ25" s="1"/>
     </row>
     <row r="26" spans="1:69" ht="15">
-      <c r="A26" s="123" t="s">
+      <c r="A26" s="109" t="s">
         <v>397</v>
       </c>
-      <c r="B26" s="123"/>
-      <c r="C26" s="123"/>
-      <c r="D26" s="123"/>
-      <c r="E26" s="123"/>
-      <c r="F26" s="123"/>
-      <c r="G26" s="123"/>
-      <c r="H26" s="123"/>
+      <c r="B26" s="109"/>
+      <c r="C26" s="109"/>
+      <c r="D26" s="109"/>
+      <c r="E26" s="109"/>
+      <c r="F26" s="109"/>
+      <c r="G26" s="109"/>
+      <c r="H26" s="109"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -45344,16 +45399,16 @@
       <c r="BQ26" s="1"/>
     </row>
     <row r="27" spans="1:69" ht="15">
-      <c r="A27" s="108" t="s">
+      <c r="A27" s="116" t="s">
         <v>398</v>
       </c>
-      <c r="B27" s="109"/>
-      <c r="C27" s="109"/>
-      <c r="D27" s="109"/>
-      <c r="E27" s="109"/>
-      <c r="F27" s="109"/>
-      <c r="G27" s="109"/>
-      <c r="H27" s="110"/>
+      <c r="B27" s="117"/>
+      <c r="C27" s="117"/>
+      <c r="D27" s="117"/>
+      <c r="E27" s="117"/>
+      <c r="F27" s="117"/>
+      <c r="G27" s="117"/>
+      <c r="H27" s="118"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -45417,14 +45472,14 @@
       <c r="BQ27" s="1"/>
     </row>
     <row r="28" spans="1:69" ht="15">
-      <c r="A28" s="111"/>
-      <c r="B28" s="112"/>
-      <c r="C28" s="112"/>
-      <c r="D28" s="112"/>
-      <c r="E28" s="112"/>
-      <c r="F28" s="112"/>
-      <c r="G28" s="112"/>
-      <c r="H28" s="113"/>
+      <c r="A28" s="119"/>
+      <c r="B28" s="120"/>
+      <c r="C28" s="120"/>
+      <c r="D28" s="120"/>
+      <c r="E28" s="120"/>
+      <c r="F28" s="120"/>
+      <c r="G28" s="120"/>
+      <c r="H28" s="121"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -45488,14 +45543,14 @@
       <c r="BQ28" s="1"/>
     </row>
     <row r="29" spans="1:69" ht="15">
-      <c r="A29" s="111"/>
-      <c r="B29" s="112"/>
-      <c r="C29" s="112"/>
-      <c r="D29" s="112"/>
-      <c r="E29" s="112"/>
-      <c r="F29" s="112"/>
-      <c r="G29" s="112"/>
-      <c r="H29" s="113"/>
+      <c r="A29" s="119"/>
+      <c r="B29" s="120"/>
+      <c r="C29" s="120"/>
+      <c r="D29" s="120"/>
+      <c r="E29" s="120"/>
+      <c r="F29" s="120"/>
+      <c r="G29" s="120"/>
+      <c r="H29" s="121"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -45559,14 +45614,14 @@
       <c r="BQ29" s="1"/>
     </row>
     <row r="30" spans="1:69" ht="15">
-      <c r="A30" s="114"/>
-      <c r="B30" s="115"/>
-      <c r="C30" s="115"/>
-      <c r="D30" s="115"/>
-      <c r="E30" s="115"/>
-      <c r="F30" s="115"/>
-      <c r="G30" s="115"/>
-      <c r="H30" s="116"/>
+      <c r="A30" s="122"/>
+      <c r="B30" s="123"/>
+      <c r="C30" s="123"/>
+      <c r="D30" s="123"/>
+      <c r="E30" s="123"/>
+      <c r="F30" s="123"/>
+      <c r="G30" s="123"/>
+      <c r="H30" s="124"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -50622,12 +50677,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="124" t="s">
+      <c r="A1" s="108" t="s">
         <v>399</v>
       </c>
-      <c r="B1" s="124"/>
-      <c r="C1" s="124"/>
-      <c r="D1" s="124"/>
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
       <c r="E1" s="107"/>
       <c r="F1" s="107"/>
       <c r="G1" s="107"/>

</xml_diff>

<commit_message>
Log July 4 project work
</commit_message>
<xml_diff>
--- a/gantt.xlsx
+++ b/gantt.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\mechanical-technical-document-evaluation-harness\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E51EF632-F772-486E-AC30-B7656800CD25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B9C5C5B-08F9-4EF3-A1ED-6328DF04849A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Start Here" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="431">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1001" uniqueCount="432">
   <si>
     <t>Mechanical Technical Document Evaluation Harness — Baseline Control Plan</t>
   </si>
@@ -499,6 +499,12 @@
     <t>-</t>
   </si>
   <si>
+    <t>Complete</t>
+  </si>
+  <si>
+    <t>Completed before baseline start on 2026-06-28. Python 3.14.2 virtual environment active; baseline tests passed.</t>
+  </si>
+  <si>
     <t>0.2</t>
   </si>
   <si>
@@ -508,6 +514,9 @@
     <t>Repository pushed; main branch protected by working practice</t>
   </si>
   <si>
+    <t>Completed 2026-06-30. Local Git initialized, baseline commit created, GitHub origin configured, and main pushed successfully. Actual time was not separately logged.</t>
+  </si>
+  <si>
     <t>0.3</t>
   </si>
   <si>
@@ -515,6 +524,12 @@
   </si>
   <si>
     <t>One-page architecture walkthrough in own words</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>Repository layout, README, CLI commands, and MECH-001 summary reviewed. Full four-schema walkthrough and concise architecture explanation remain.</t>
   </si>
   <si>
     <t>0.4</t>
@@ -536,6 +551,9 @@
   </si>
   <si>
     <t>Updated weekly control sheet and issue notes</t>
+  </si>
+  <si>
+    <t>Week 1 control update completed. Actual time is recorded only where explicitly tracked.</t>
   </si>
   <si>
     <t>0.6</t>
@@ -628,6 +646,9 @@
     <t>Three clean feature branches and one intentional recovery exercise</t>
   </si>
   <si>
+    <t>Started early. Created feature/test-unknown-case and added the first controlled test change. Push/PR/merge evidence and two more branches plus recovery exercise remain.</t>
+  </si>
+  <si>
     <t>2.2</t>
   </si>
   <si>
@@ -644,6 +665,9 @@
   </si>
   <si>
     <t>Positive and negative cases run locally</t>
+  </si>
+  <si>
+    <t>Completed early on 2026-06-30. Added a negative CLI integration test; 20 tests pass locally. Actual time was not separately logged.</t>
   </si>
   <si>
     <t>2.4</t>
@@ -1294,31 +1318,10 @@
     <t>Informs authentic mechanical document, QA/QC, revision, maintenance, and technical-record workflow selection.</t>
   </si>
   <si>
-    <t>Complete</t>
+    <t>Started early on 2026-07-04. Added targeted load_case_by_id, updated CLI inspect to load one case directly, added positive and negative regression tests, fixed inspect output formatting, merged PR #2, and confirmed 22 tests pass.</t>
   </si>
   <si>
-    <t>Completed before baseline start on 2026-06-28. Python 3.14.2 virtual environment active; baseline tests passed.</t>
-  </si>
-  <si>
-    <t>Completed 2026-06-30. Local Git initialized, baseline commit created, GitHub origin configured, and main pushed successfully. Actual time was not separately logged.</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>Repository layout, README, CLI commands, and MECH-001 summary reviewed. Full four-schema walkthrough and concise architecture explanation remain.</t>
-  </si>
-  <si>
-    <t>Week 1 control update completed. Actual time is recorded only where explicitly tracked.</t>
-  </si>
-  <si>
-    <t>Started early. Created feature/test-unknown-case and added the first controlled test change. Push/PR/merge evidence and two more branches plus recovery exercise remain.</t>
-  </si>
-  <si>
-    <t>Completed early on 2026-06-30. Added a negative CLI integration test; 20 tests pass locally. Actual time was not separately logged.</t>
-  </si>
-  <si>
-    <t>Completed Python environment and Git/GitHub baseline; validated all 3 seed cases; inspected MECH-001; reached 20 passing tests. Only 1.5 hours were explicitly time-tracked, so other completed work remains unallocated in Actual Hours.</t>
+    <t>Completed Python environment and Git/GitHub baseline; validated all 3 seed cases; inspected MECH-001; reached 20 passing tests. On 2026-07-04, added targeted case loading by ID, merged PR #2, and reached 22 passing tests. Week 1 actual hours now include the previously recorded 1.5 h plus today's 0.62 h.</t>
   </si>
 </sst>
 </file>
@@ -1573,7 +1576,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="132">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1884,29 +1887,14 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1935,6 +1923,15 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1942,6 +1939,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2393,7 +2405,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-385B-41B8-85CE-A9C9AFF7D0EE}"/>
+              <c16:uniqueId val="{00000000-32C8-4FB4-8EF5-94845203858B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2574,8 +2586,8 @@
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="52"/>
-                <c:pt idx="0">
-                  <c:v>1.5</c:v>
+                <c:pt idx="0" formatCode="0.00">
+                  <c:v>2.12</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2583,7 +2595,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-385B-41B8-85CE-A9C9AFF7D0EE}"/>
+              <c16:uniqueId val="{00000001-32C8-4FB4-8EF5-94845203858B}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2780,7 +2792,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-E919-4C75-A1FE-46BAE985CCA2}"/>
+              <c16:uniqueId val="{00000000-30A7-4CBF-8CD3-77CE41B2D3FC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -3157,16 +3169,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="30" customHeight="1">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="127" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -3308,13 +3320,13 @@
         <v>46202</v>
       </c>
       <c r="C3" s="1"/>
-      <c r="D3" s="109" t="s">
+      <c r="D3" s="126" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="109"/>
-      <c r="F3" s="109"/>
-      <c r="G3" s="109"/>
-      <c r="H3" s="109"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -3388,12 +3400,12 @@
       <c r="D4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="110" t="s">
+      <c r="E4" s="128" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="111"/>
-      <c r="G4" s="111"/>
-      <c r="H4" s="112"/>
+      <c r="F4" s="129"/>
+      <c r="G4" s="129"/>
+      <c r="H4" s="130"/>
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
@@ -3467,12 +3479,12 @@
       <c r="D5" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="113" t="s">
+      <c r="E5" s="120" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="114"/>
-      <c r="G5" s="114"/>
-      <c r="H5" s="115"/>
+      <c r="F5" s="121"/>
+      <c r="G5" s="121"/>
+      <c r="H5" s="122"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
@@ -3546,12 +3558,12 @@
       <c r="D6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E6" s="113" t="s">
+      <c r="E6" s="120" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="114"/>
-      <c r="G6" s="114"/>
-      <c r="H6" s="115"/>
+      <c r="F6" s="121"/>
+      <c r="G6" s="121"/>
+      <c r="H6" s="122"/>
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
@@ -3625,12 +3637,12 @@
       <c r="D7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="113" t="s">
+      <c r="E7" s="120" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="114"/>
-      <c r="G7" s="114"/>
-      <c r="H7" s="115"/>
+      <c r="F7" s="121"/>
+      <c r="G7" s="121"/>
+      <c r="H7" s="122"/>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
@@ -3704,12 +3716,12 @@
       <c r="D8" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E8" s="113" t="s">
+      <c r="E8" s="120" t="s">
         <v>20</v>
       </c>
-      <c r="F8" s="114"/>
-      <c r="G8" s="114"/>
-      <c r="H8" s="115"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="121"/>
+      <c r="H8" s="122"/>
       <c r="I8" s="1"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
@@ -3783,12 +3795,12 @@
       <c r="D9" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="113" t="s">
+      <c r="E9" s="120" t="s">
         <v>23</v>
       </c>
-      <c r="F9" s="114"/>
-      <c r="G9" s="114"/>
-      <c r="H9" s="115"/>
+      <c r="F9" s="121"/>
+      <c r="G9" s="121"/>
+      <c r="H9" s="122"/>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
@@ -3862,12 +3874,12 @@
       <c r="D10" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="E10" s="125" t="s">
+      <c r="E10" s="123" t="s">
         <v>27</v>
       </c>
-      <c r="F10" s="126"/>
-      <c r="G10" s="126"/>
-      <c r="H10" s="127"/>
+      <c r="F10" s="124"/>
+      <c r="G10" s="124"/>
+      <c r="H10" s="125"/>
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
@@ -4148,16 +4160,16 @@
       <c r="BQ13" s="1"/>
     </row>
     <row r="14" spans="1:69" ht="15">
-      <c r="A14" s="109" t="s">
+      <c r="A14" s="126" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="109"/>
-      <c r="C14" s="109"/>
-      <c r="D14" s="109"/>
-      <c r="E14" s="109"/>
-      <c r="F14" s="109"/>
-      <c r="G14" s="109"/>
-      <c r="H14" s="109"/>
+      <c r="B14" s="126"/>
+      <c r="C14" s="126"/>
+      <c r="D14" s="126"/>
+      <c r="E14" s="126"/>
+      <c r="F14" s="126"/>
+      <c r="G14" s="126"/>
+      <c r="H14" s="126"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -4221,16 +4233,16 @@
       <c r="BQ14" s="1"/>
     </row>
     <row r="15" spans="1:69" ht="15">
-      <c r="A15" s="116" t="s">
+      <c r="A15" s="111" t="s">
         <v>31</v>
       </c>
-      <c r="B15" s="117"/>
-      <c r="C15" s="117"/>
-      <c r="D15" s="117"/>
-      <c r="E15" s="117"/>
-      <c r="F15" s="117"/>
-      <c r="G15" s="117"/>
-      <c r="H15" s="118"/>
+      <c r="B15" s="112"/>
+      <c r="C15" s="112"/>
+      <c r="D15" s="112"/>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
+      <c r="G15" s="112"/>
+      <c r="H15" s="113"/>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
@@ -4294,14 +4306,14 @@
       <c r="BQ15" s="1"/>
     </row>
     <row r="16" spans="1:69" ht="15">
-      <c r="A16" s="119"/>
-      <c r="B16" s="120"/>
-      <c r="C16" s="120"/>
-      <c r="D16" s="120"/>
-      <c r="E16" s="120"/>
-      <c r="F16" s="120"/>
-      <c r="G16" s="120"/>
-      <c r="H16" s="121"/>
+      <c r="A16" s="114"/>
+      <c r="B16" s="115"/>
+      <c r="C16" s="115"/>
+      <c r="D16" s="115"/>
+      <c r="E16" s="115"/>
+      <c r="F16" s="115"/>
+      <c r="G16" s="115"/>
+      <c r="H16" s="116"/>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
@@ -4365,14 +4377,14 @@
       <c r="BQ16" s="1"/>
     </row>
     <row r="17" spans="1:69" ht="15">
-      <c r="A17" s="119"/>
-      <c r="B17" s="120"/>
-      <c r="C17" s="120"/>
-      <c r="D17" s="120"/>
-      <c r="E17" s="120"/>
-      <c r="F17" s="120"/>
-      <c r="G17" s="120"/>
-      <c r="H17" s="121"/>
+      <c r="A17" s="114"/>
+      <c r="B17" s="115"/>
+      <c r="C17" s="115"/>
+      <c r="D17" s="115"/>
+      <c r="E17" s="115"/>
+      <c r="F17" s="115"/>
+      <c r="G17" s="115"/>
+      <c r="H17" s="116"/>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
@@ -4436,14 +4448,14 @@
       <c r="BQ17" s="1"/>
     </row>
     <row r="18" spans="1:69" ht="15">
-      <c r="A18" s="122"/>
-      <c r="B18" s="123"/>
-      <c r="C18" s="123"/>
-      <c r="D18" s="123"/>
-      <c r="E18" s="123"/>
-      <c r="F18" s="123"/>
-      <c r="G18" s="123"/>
-      <c r="H18" s="124"/>
+      <c r="A18" s="117"/>
+      <c r="B18" s="118"/>
+      <c r="C18" s="118"/>
+      <c r="D18" s="118"/>
+      <c r="E18" s="118"/>
+      <c r="F18" s="118"/>
+      <c r="G18" s="118"/>
+      <c r="H18" s="119"/>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
@@ -10330,17 +10342,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="D3:H3"/>
+    <mergeCell ref="E4:H4"/>
+    <mergeCell ref="E5:H5"/>
+    <mergeCell ref="E6:H6"/>
     <mergeCell ref="A15:H18"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="E9:H9"/>
     <mergeCell ref="E10:H10"/>
     <mergeCell ref="A14:H14"/>
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="D3:H3"/>
-    <mergeCell ref="E4:H4"/>
-    <mergeCell ref="E5:H5"/>
-    <mergeCell ref="E6:H6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10361,28 +10373,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="108" t="s">
+      <c r="A1" s="127" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="108"/>
-      <c r="M1" s="108"/>
-      <c r="N1" s="108"/>
-      <c r="O1" s="108"/>
-      <c r="P1" s="108"/>
-      <c r="Q1" s="108"/>
-      <c r="R1" s="108"/>
-      <c r="S1" s="108"/>
-      <c r="T1" s="108"/>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
+      <c r="M1" s="127"/>
+      <c r="N1" s="127"/>
+      <c r="O1" s="127"/>
+      <c r="P1" s="127"/>
+      <c r="Q1" s="127"/>
+      <c r="R1" s="127"/>
+      <c r="S1" s="127"/>
+      <c r="T1" s="127"/>
       <c r="U1" s="107"/>
       <c r="V1" s="107"/>
       <c r="W1" s="107"/>
@@ -11301,10 +11313,10 @@
       <c r="BQ10" s="1"/>
     </row>
     <row r="11" spans="1:69" ht="15">
-      <c r="A11" s="128" t="s">
+      <c r="A11" s="131" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="129"/>
+      <c r="B11" s="132"/>
       <c r="C11" s="42">
         <v>576</v>
       </c>
@@ -17723,35 +17735,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="15">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="126" t="s">
         <v>80</v>
       </c>
-      <c r="B1" s="109"/>
+      <c r="B1" s="126"/>
       <c r="C1" s="45">
         <v>46202</v>
       </c>
-      <c r="D1" s="109" t="s">
+      <c r="D1" s="126" t="s">
         <v>81</v>
       </c>
-      <c r="E1" s="109"/>
-      <c r="F1" s="109"/>
+      <c r="E1" s="126"/>
+      <c r="F1" s="126"/>
       <c r="G1" s="4">
         <v>576</v>
       </c>
-      <c r="H1" s="109" t="s">
+      <c r="H1" s="126" t="s">
         <v>82</v>
       </c>
-      <c r="I1" s="109"/>
-      <c r="J1" s="109"/>
-      <c r="K1" s="109"/>
-      <c r="L1" s="109" t="s">
+      <c r="I1" s="126"/>
+      <c r="J1" s="126"/>
+      <c r="K1" s="126"/>
+      <c r="L1" s="126" t="s">
         <v>83</v>
       </c>
-      <c r="M1" s="109"/>
-      <c r="N1" s="109"/>
-      <c r="O1" s="109"/>
-      <c r="P1" s="109"/>
-      <c r="Q1" s="109"/>
+      <c r="M1" s="126"/>
+      <c r="N1" s="126"/>
+      <c r="O1" s="126"/>
+      <c r="P1" s="126"/>
+      <c r="Q1" s="126"/>
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
       <c r="T1" s="1"/>
@@ -17877,27 +17889,27 @@
       <c r="BQ2" s="1"/>
     </row>
     <row r="3" spans="1:69" ht="15">
-      <c r="A3" s="130" t="s">
+      <c r="A3" s="133" t="s">
         <v>84</v>
       </c>
-      <c r="B3" s="130"/>
-      <c r="C3" s="131" t="s">
+      <c r="B3" s="133"/>
+      <c r="C3" s="134" t="s">
         <v>85</v>
       </c>
-      <c r="D3" s="131"/>
-      <c r="E3" s="131"/>
-      <c r="F3" s="131"/>
-      <c r="G3" s="131"/>
-      <c r="H3" s="131"/>
-      <c r="I3" s="131"/>
-      <c r="J3" s="131"/>
-      <c r="K3" s="131"/>
-      <c r="L3" s="131"/>
-      <c r="M3" s="131"/>
-      <c r="N3" s="131"/>
-      <c r="O3" s="131"/>
-      <c r="P3" s="131"/>
-      <c r="Q3" s="131"/>
+      <c r="D3" s="134"/>
+      <c r="E3" s="134"/>
+      <c r="F3" s="134"/>
+      <c r="G3" s="134"/>
+      <c r="H3" s="134"/>
+      <c r="I3" s="134"/>
+      <c r="J3" s="134"/>
+      <c r="K3" s="134"/>
+      <c r="L3" s="134"/>
+      <c r="M3" s="134"/>
+      <c r="N3" s="134"/>
+      <c r="O3" s="134"/>
+      <c r="P3" s="134"/>
+      <c r="Q3" s="134"/>
       <c r="R3" s="1"/>
       <c r="S3" s="1"/>
       <c r="T3" s="1"/>
@@ -18373,7 +18385,7 @@
         <v>46208</v>
       </c>
       <c r="L6" s="47" t="s">
-        <v>422</v>
+        <v>157</v>
       </c>
       <c r="M6" s="49">
         <v>1</v>
@@ -18390,7 +18402,7 @@
         <v>0</v>
       </c>
       <c r="Q6" s="25" t="s">
-        <v>423</v>
+        <v>158</v>
       </c>
       <c r="R6" s="50" t="s">
         <v>57</v>
@@ -18449,16 +18461,16 @@
     </row>
     <row r="7" spans="1:69" ht="42" customHeight="1">
       <c r="A7" s="20" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="B7" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>153</v>
@@ -18485,7 +18497,7 @@
         <v>46208</v>
       </c>
       <c r="L7" s="47" t="s">
-        <v>422</v>
+        <v>157</v>
       </c>
       <c r="M7" s="49">
         <v>1</v>
@@ -18500,7 +18512,7 @@
         <v>0</v>
       </c>
       <c r="Q7" s="25" t="s">
-        <v>424</v>
+        <v>162</v>
       </c>
       <c r="R7" s="50" t="s">
         <v>57</v>
@@ -18559,16 +18571,16 @@
     </row>
     <row r="8" spans="1:69" ht="42" customHeight="1">
       <c r="A8" s="20" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B8" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C8" s="22" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D8" s="22" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>153</v>
@@ -18595,7 +18607,7 @@
         <v>46215</v>
       </c>
       <c r="L8" s="47" t="s">
-        <v>425</v>
+        <v>166</v>
       </c>
       <c r="M8" s="49">
         <v>0.5</v>
@@ -18610,7 +18622,7 @@
         <v>2</v>
       </c>
       <c r="Q8" s="25" t="s">
-        <v>426</v>
+        <v>167</v>
       </c>
       <c r="R8" s="55" t="s">
         <v>57</v>
@@ -18671,19 +18683,19 @@
     </row>
     <row r="9" spans="1:69" ht="42" customHeight="1">
       <c r="A9" s="20" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B9" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C9" s="22" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="E9" s="22" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="F9" s="47">
         <v>4</v>
@@ -18707,7 +18719,7 @@
         <v>46215</v>
       </c>
       <c r="L9" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M9" s="49">
         <v>0</v>
@@ -18779,19 +18791,19 @@
     </row>
     <row r="10" spans="1:69" ht="42" customHeight="1">
       <c r="A10" s="20" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B10" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C10" s="22" t="s">
+        <v>173</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>174</v>
+      </c>
+      <c r="E10" s="22" t="s">
         <v>168</v>
-      </c>
-      <c r="D10" s="22" t="s">
-        <v>169</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>163</v>
       </c>
       <c r="F10" s="47">
         <v>12</v>
@@ -18815,7 +18827,7 @@
         <v>46565</v>
       </c>
       <c r="L10" s="47" t="s">
-        <v>425</v>
+        <v>166</v>
       </c>
       <c r="M10" s="49">
         <v>0.02</v>
@@ -18830,7 +18842,7 @@
         <v>11.76</v>
       </c>
       <c r="Q10" s="25" t="s">
-        <v>427</v>
+        <v>175</v>
       </c>
       <c r="R10" s="55" t="s">
         <v>57</v>
@@ -18991,19 +19003,19 @@
     </row>
     <row r="11" spans="1:69" ht="42" customHeight="1">
       <c r="A11" s="20" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="B11" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="D11" s="22" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="E11" s="22" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F11" s="47">
         <v>6</v>
@@ -19027,7 +19039,7 @@
         <v>46565</v>
       </c>
       <c r="L11" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M11" s="49">
         <v>0</v>
@@ -19195,19 +19207,19 @@
     </row>
     <row r="12" spans="1:69" ht="42" customHeight="1">
       <c r="A12" s="20" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B12" s="21" t="s">
         <v>54</v>
       </c>
       <c r="C12" s="22" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="D12" s="22" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="E12" s="22" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="F12" s="47">
         <v>6</v>
@@ -19231,7 +19243,7 @@
         <v>46565</v>
       </c>
       <c r="L12" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M12" s="49">
         <v>0</v>
@@ -19389,19 +19401,19 @@
     </row>
     <row r="13" spans="1:69" ht="42" customHeight="1">
       <c r="A13" s="20" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="B13" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F13" s="47">
         <v>8</v>
@@ -19425,7 +19437,7 @@
         <v>46222</v>
       </c>
       <c r="L13" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M13" s="49">
         <v>0</v>
@@ -19497,19 +19509,19 @@
     </row>
     <row r="14" spans="1:69" ht="42" customHeight="1">
       <c r="A14" s="20" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="B14" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C14" s="22" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="D14" s="22" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="E14" s="22" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="F14" s="47">
         <v>6</v>
@@ -19533,7 +19545,7 @@
         <v>46229</v>
       </c>
       <c r="L14" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M14" s="49">
         <v>0</v>
@@ -19607,19 +19619,19 @@
     </row>
     <row r="15" spans="1:69" ht="42" customHeight="1">
       <c r="A15" s="20" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B15" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C15" s="22" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="E15" s="22" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="F15" s="47">
         <v>14</v>
@@ -19643,7 +19655,7 @@
         <v>46236</v>
       </c>
       <c r="L15" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M15" s="49">
         <v>0</v>
@@ -19717,19 +19729,19 @@
     </row>
     <row r="16" spans="1:69" ht="42" customHeight="1">
       <c r="A16" s="20" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B16" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C16" s="22" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="E16" s="22" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="F16" s="47">
         <v>18</v>
@@ -19753,7 +19765,7 @@
         <v>46250</v>
       </c>
       <c r="L16" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M16" s="49">
         <v>0</v>
@@ -19829,19 +19841,19 @@
     </row>
     <row r="17" spans="1:69" ht="42" customHeight="1">
       <c r="A17" s="20" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B17" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C17" s="22" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="F17" s="47">
         <v>6</v>
@@ -19865,7 +19877,7 @@
         <v>46257</v>
       </c>
       <c r="L17" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M17" s="49">
         <v>0</v>
@@ -19939,19 +19951,19 @@
     </row>
     <row r="18" spans="1:69" ht="42" customHeight="1">
       <c r="A18" s="20" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B18" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C18" s="22" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="E18" s="22" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="F18" s="47">
         <v>6</v>
@@ -19975,7 +19987,7 @@
         <v>46257</v>
       </c>
       <c r="L18" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M18" s="49">
         <v>0</v>
@@ -20047,19 +20059,19 @@
     </row>
     <row r="19" spans="1:69" ht="42" customHeight="1">
       <c r="A19" s="20" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B19" s="27" t="s">
         <v>58</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="F19" s="47">
         <v>6</v>
@@ -20083,7 +20095,7 @@
         <v>46264</v>
       </c>
       <c r="L19" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M19" s="49">
         <v>0</v>
@@ -20155,19 +20167,19 @@
     </row>
     <row r="20" spans="1:69" ht="42" customHeight="1">
       <c r="A20" s="20" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="B20" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="E20" s="22" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="F20" s="47">
         <v>10</v>
@@ -20191,7 +20203,7 @@
         <v>46271</v>
       </c>
       <c r="L20" s="47" t="s">
-        <v>425</v>
+        <v>166</v>
       </c>
       <c r="M20" s="49">
         <v>0.2</v>
@@ -20206,7 +20218,7 @@
         <v>8</v>
       </c>
       <c r="Q20" s="25" t="s">
-        <v>428</v>
+        <v>206</v>
       </c>
       <c r="R20" s="57"/>
       <c r="S20" s="53"/>
@@ -20265,19 +20277,19 @@
     </row>
     <row r="21" spans="1:69" ht="42" customHeight="1">
       <c r="A21" s="20" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="B21" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C21" s="22" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="E21" s="22" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="F21" s="47">
         <v>12</v>
@@ -20303,19 +20315,23 @@
       <c r="L21" s="47" t="s">
         <v>166</v>
       </c>
-      <c r="M21" s="49">
-        <v>0</v>
-      </c>
-      <c r="N21" s="47"/>
-      <c r="O21" s="47" t="str">
+      <c r="M21" s="108">
+        <v>0.15</v>
+      </c>
+      <c r="N21" s="109">
+        <v>0.62</v>
+      </c>
+      <c r="O21" s="109">
         <f t="shared" si="3"/>
-        <v/>
+        <v>-11.38</v>
       </c>
       <c r="P21" s="47">
         <f t="shared" si="4"/>
-        <v>12</v>
-      </c>
-      <c r="Q21" s="25"/>
+        <v>10.199999999999999</v>
+      </c>
+      <c r="Q21" s="25" t="s">
+        <v>430</v>
+      </c>
       <c r="R21" s="57"/>
       <c r="S21" s="53"/>
       <c r="T21" s="53"/>
@@ -20375,19 +20391,19 @@
     </row>
     <row r="22" spans="1:69" ht="42" customHeight="1">
       <c r="A22" s="20" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="B22" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="E22" s="22" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="F22" s="47">
         <v>14</v>
@@ -20411,7 +20427,7 @@
         <v>46285</v>
       </c>
       <c r="L22" s="47" t="s">
-        <v>422</v>
+        <v>157</v>
       </c>
       <c r="M22" s="49">
         <v>1</v>
@@ -20426,7 +20442,7 @@
         <v>0</v>
       </c>
       <c r="Q22" s="25" t="s">
-        <v>429</v>
+        <v>213</v>
       </c>
       <c r="R22" s="57"/>
       <c r="S22" s="53"/>
@@ -20487,19 +20503,19 @@
     </row>
     <row r="23" spans="1:69" ht="42" customHeight="1">
       <c r="A23" s="20" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="B23" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C23" s="22" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="E23" s="22" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="F23" s="47">
         <v>10</v>
@@ -20523,7 +20539,7 @@
         <v>46292</v>
       </c>
       <c r="L23" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M23" s="49">
         <v>0</v>
@@ -20597,19 +20613,19 @@
     </row>
     <row r="24" spans="1:69" ht="42" customHeight="1">
       <c r="A24" s="20" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="B24" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C24" s="22" t="s">
+        <v>218</v>
+      </c>
+      <c r="D24" s="22" t="s">
+        <v>219</v>
+      </c>
+      <c r="E24" s="22" t="s">
         <v>210</v>
-      </c>
-      <c r="D24" s="22" t="s">
-        <v>211</v>
-      </c>
-      <c r="E24" s="22" t="s">
-        <v>203</v>
       </c>
       <c r="F24" s="47">
         <v>10</v>
@@ -20633,7 +20649,7 @@
         <v>46299</v>
       </c>
       <c r="L24" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M24" s="49">
         <v>0</v>
@@ -20707,19 +20723,19 @@
     </row>
     <row r="25" spans="1:69" ht="42" customHeight="1">
       <c r="A25" s="20" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="B25" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="D25" s="22" t="s">
+        <v>222</v>
+      </c>
+      <c r="E25" s="22" t="s">
         <v>214</v>
-      </c>
-      <c r="E25" s="22" t="s">
-        <v>206</v>
       </c>
       <c r="F25" s="47">
         <v>8</v>
@@ -20743,7 +20759,7 @@
         <v>46306</v>
       </c>
       <c r="L25" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M25" s="49">
         <v>0</v>
@@ -20817,19 +20833,19 @@
     </row>
     <row r="26" spans="1:69" ht="42" customHeight="1">
       <c r="A26" s="20" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="B26" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C26" s="22" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="D26" s="22" t="s">
+        <v>225</v>
+      </c>
+      <c r="E26" s="22" t="s">
         <v>217</v>
-      </c>
-      <c r="E26" s="22" t="s">
-        <v>209</v>
       </c>
       <c r="F26" s="47">
         <v>4</v>
@@ -20853,7 +20869,7 @@
         <v>46306</v>
       </c>
       <c r="L26" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M26" s="49">
         <v>0</v>
@@ -20925,19 +20941,19 @@
     </row>
     <row r="27" spans="1:69" ht="42" customHeight="1">
       <c r="A27" s="20" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="B27" s="30" t="s">
         <v>61</v>
       </c>
       <c r="C27" s="22" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="D27" s="22" t="s">
+        <v>228</v>
+      </c>
+      <c r="E27" s="22" t="s">
         <v>220</v>
-      </c>
-      <c r="E27" s="22" t="s">
-        <v>212</v>
       </c>
       <c r="F27" s="47">
         <v>4</v>
@@ -20961,7 +20977,7 @@
         <v>46313</v>
       </c>
       <c r="L27" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M27" s="49">
         <v>0</v>
@@ -21033,19 +21049,19 @@
     </row>
     <row r="28" spans="1:69" ht="42" customHeight="1">
       <c r="A28" s="20" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="B28" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C28" s="22" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="D28" s="22" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="E28" s="22" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="F28" s="47">
         <v>18</v>
@@ -21069,7 +21085,7 @@
         <v>46327</v>
       </c>
       <c r="L28" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M28" s="49">
         <v>0</v>
@@ -21143,19 +21159,19 @@
     </row>
     <row r="29" spans="1:69" ht="42" customHeight="1">
       <c r="A29" s="20" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="B29" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C29" s="22" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="D29" s="22" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="E29" s="22" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="F29" s="47">
         <v>12</v>
@@ -21179,7 +21195,7 @@
         <v>46334</v>
       </c>
       <c r="L29" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M29" s="49">
         <v>0</v>
@@ -21253,19 +21269,19 @@
     </row>
     <row r="30" spans="1:69" ht="42" customHeight="1">
       <c r="A30" s="20" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="B30" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="F30" s="47">
         <v>12</v>
@@ -21289,7 +21305,7 @@
         <v>46341</v>
       </c>
       <c r="L30" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M30" s="49">
         <v>0</v>
@@ -21363,19 +21379,19 @@
     </row>
     <row r="31" spans="1:69" ht="42" customHeight="1">
       <c r="A31" s="20" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="B31" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C31" s="22" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D31" s="22" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="F31" s="47">
         <v>8</v>
@@ -21399,7 +21415,7 @@
         <v>46341</v>
       </c>
       <c r="L31" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M31" s="49">
         <v>0</v>
@@ -21471,19 +21487,19 @@
     </row>
     <row r="32" spans="1:69" ht="42" customHeight="1">
       <c r="A32" s="20" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="B32" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="E32" s="22" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="F32" s="47">
         <v>10</v>
@@ -21507,7 +21523,7 @@
         <v>46348</v>
       </c>
       <c r="L32" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M32" s="49">
         <v>0</v>
@@ -21579,19 +21595,19 @@
     </row>
     <row r="33" spans="1:69" ht="42" customHeight="1">
       <c r="A33" s="20" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="B33" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>238</v>
+        <v>246</v>
       </c>
       <c r="E33" s="22" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="F33" s="47">
         <v>10</v>
@@ -21615,7 +21631,7 @@
         <v>46355</v>
       </c>
       <c r="L33" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M33" s="49">
         <v>0</v>
@@ -21689,19 +21705,19 @@
     </row>
     <row r="34" spans="1:69" ht="42" customHeight="1">
       <c r="A34" s="20" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="B34" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>240</v>
+        <v>248</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>241</v>
+        <v>249</v>
       </c>
       <c r="E34" s="22" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="F34" s="47">
         <v>10</v>
@@ -21725,7 +21741,7 @@
         <v>46362</v>
       </c>
       <c r="L34" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M34" s="49">
         <v>0</v>
@@ -21799,19 +21815,19 @@
     </row>
     <row r="35" spans="1:69" ht="42" customHeight="1">
       <c r="A35" s="20" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="B35" s="32" t="s">
         <v>64</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>243</v>
+        <v>251</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>244</v>
+        <v>252</v>
       </c>
       <c r="E35" s="22" t="s">
-        <v>239</v>
+        <v>247</v>
       </c>
       <c r="F35" s="47">
         <v>8</v>
@@ -21835,7 +21851,7 @@
         <v>46369</v>
       </c>
       <c r="L35" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M35" s="49">
         <v>0</v>
@@ -21907,19 +21923,19 @@
     </row>
     <row r="36" spans="1:69" ht="42" customHeight="1">
       <c r="A36" s="20" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="B36" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>246</v>
+        <v>254</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>247</v>
+        <v>255</v>
       </c>
       <c r="E36" s="22" t="s">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="F36" s="47">
         <v>8</v>
@@ -21943,7 +21959,7 @@
         <v>46376</v>
       </c>
       <c r="L36" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M36" s="49">
         <v>0</v>
@@ -22015,19 +22031,19 @@
     </row>
     <row r="37" spans="1:69" ht="42" customHeight="1">
       <c r="A37" s="20" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="B37" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>249</v>
+        <v>257</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>250</v>
+        <v>258</v>
       </c>
       <c r="E37" s="22" t="s">
-        <v>245</v>
+        <v>253</v>
       </c>
       <c r="F37" s="47">
         <v>10</v>
@@ -22051,7 +22067,7 @@
         <v>46383</v>
       </c>
       <c r="L37" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M37" s="49">
         <v>0</v>
@@ -22125,19 +22141,19 @@
     </row>
     <row r="38" spans="1:69" ht="42" customHeight="1">
       <c r="A38" s="20" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="B38" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C38" s="22" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
       <c r="D38" s="22" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="E38" s="22" t="s">
-        <v>248</v>
+        <v>256</v>
       </c>
       <c r="F38" s="47">
         <v>18</v>
@@ -22161,7 +22177,7 @@
         <v>46397</v>
       </c>
       <c r="L38" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M38" s="49">
         <v>0</v>
@@ -22237,19 +22253,19 @@
     </row>
     <row r="39" spans="1:69" ht="42" customHeight="1">
       <c r="A39" s="20" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="B39" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="E39" s="22" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
       <c r="F39" s="47">
         <v>14</v>
@@ -22273,7 +22289,7 @@
         <v>46404</v>
       </c>
       <c r="L39" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M39" s="49">
         <v>0</v>
@@ -22347,19 +22363,19 @@
     </row>
     <row r="40" spans="1:69" ht="42" customHeight="1">
       <c r="A40" s="20" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="B40" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C40" s="22" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="D40" s="22" t="s">
+        <v>267</v>
+      </c>
+      <c r="E40" s="22" t="s">
         <v>259</v>
-      </c>
-      <c r="E40" s="22" t="s">
-        <v>251</v>
       </c>
       <c r="F40" s="47">
         <v>14</v>
@@ -22383,7 +22399,7 @@
         <v>46411</v>
       </c>
       <c r="L40" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M40" s="49">
         <v>0</v>
@@ -22457,19 +22473,19 @@
     </row>
     <row r="41" spans="1:69" ht="42" customHeight="1">
       <c r="A41" s="20" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="B41" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C41" s="22" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="D41" s="22" t="s">
+        <v>270</v>
+      </c>
+      <c r="E41" s="22" t="s">
         <v>262</v>
-      </c>
-      <c r="E41" s="22" t="s">
-        <v>254</v>
       </c>
       <c r="F41" s="47">
         <v>20</v>
@@ -22493,7 +22509,7 @@
         <v>46418</v>
       </c>
       <c r="L41" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M41" s="49">
         <v>0</v>
@@ -22567,19 +22583,19 @@
     </row>
     <row r="42" spans="1:69" ht="42" customHeight="1">
       <c r="A42" s="20" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="B42" s="34" t="s">
         <v>67</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="E42" s="22" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="F42" s="47">
         <v>12</v>
@@ -22603,7 +22619,7 @@
         <v>46425</v>
       </c>
       <c r="L42" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M42" s="49">
         <v>0</v>
@@ -22675,19 +22691,19 @@
     </row>
     <row r="43" spans="1:69" ht="42" customHeight="1">
       <c r="A43" s="20" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="B43" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C43" s="22" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="D43" s="22" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="E43" s="22" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="F43" s="47">
         <v>10</v>
@@ -22711,7 +22727,7 @@
         <v>46432</v>
       </c>
       <c r="L43" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M43" s="49">
         <v>0</v>
@@ -22783,19 +22799,19 @@
     </row>
     <row r="44" spans="1:69" ht="42" customHeight="1">
       <c r="A44" s="20" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="B44" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C44" s="22" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="D44" s="22" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="E44" s="22" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="F44" s="47">
         <v>16</v>
@@ -22819,7 +22835,7 @@
         <v>46446</v>
       </c>
       <c r="L44" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M44" s="49">
         <v>0</v>
@@ -22893,19 +22909,19 @@
     </row>
     <row r="45" spans="1:69" ht="42" customHeight="1">
       <c r="A45" s="20" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="B45" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C45" s="22" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
       <c r="D45" s="22" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
       <c r="E45" s="22" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="F45" s="47">
         <v>12</v>
@@ -22929,7 +22945,7 @@
         <v>46453</v>
       </c>
       <c r="L45" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M45" s="49">
         <v>0</v>
@@ -23003,19 +23019,19 @@
     </row>
     <row r="46" spans="1:69" ht="42" customHeight="1">
       <c r="A46" s="20" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="B46" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C46" s="22" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
       <c r="D46" s="22" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
       <c r="E46" s="22" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="F46" s="47">
         <v>10</v>
@@ -23039,7 +23055,7 @@
         <v>46453</v>
       </c>
       <c r="L46" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M46" s="49">
         <v>0</v>
@@ -23111,19 +23127,19 @@
     </row>
     <row r="47" spans="1:69" ht="42" customHeight="1">
       <c r="A47" s="20" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="B47" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C47" s="22" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
       <c r="D47" s="22" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
       <c r="E47" s="22" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
       <c r="F47" s="47">
         <v>16</v>
@@ -23147,7 +23163,7 @@
         <v>46467</v>
       </c>
       <c r="L47" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M47" s="49">
         <v>0</v>
@@ -23221,19 +23237,19 @@
     </row>
     <row r="48" spans="1:69" ht="42" customHeight="1">
       <c r="A48" s="20" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="B48" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C48" s="22" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
       <c r="D48" s="22" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="E48" s="22" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
       <c r="F48" s="47">
         <v>14</v>
@@ -23257,7 +23273,7 @@
         <v>46474</v>
       </c>
       <c r="L48" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M48" s="49">
         <v>0</v>
@@ -23331,19 +23347,19 @@
     </row>
     <row r="49" spans="1:69" ht="42" customHeight="1">
       <c r="A49" s="20" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="B49" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C49" s="22" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
       <c r="D49" s="22" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
       <c r="E49" s="22" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
       <c r="F49" s="47">
         <v>16</v>
@@ -23367,7 +23383,7 @@
         <v>46488</v>
       </c>
       <c r="L49" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M49" s="49">
         <v>0</v>
@@ -23441,19 +23457,19 @@
     </row>
     <row r="50" spans="1:69" ht="42" customHeight="1">
       <c r="A50" s="20" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="B50" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C50" s="22" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
       <c r="D50" s="22" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
       <c r="E50" s="22" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
       <c r="F50" s="47">
         <v>10</v>
@@ -23477,7 +23493,7 @@
         <v>46495</v>
       </c>
       <c r="L50" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M50" s="49">
         <v>0</v>
@@ -23549,19 +23565,19 @@
     </row>
     <row r="51" spans="1:69" ht="42" customHeight="1">
       <c r="A51" s="20" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="B51" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C51" s="22" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
       <c r="D51" s="22" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
       <c r="E51" s="22" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
       <c r="F51" s="47">
         <v>6</v>
@@ -23585,7 +23601,7 @@
         <v>46502</v>
       </c>
       <c r="L51" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M51" s="49">
         <v>0</v>
@@ -23657,19 +23673,19 @@
     </row>
     <row r="52" spans="1:69" ht="42" customHeight="1">
       <c r="A52" s="20" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="B52" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C52" s="22" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
       <c r="D52" s="22" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
       <c r="E52" s="22" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
       <c r="F52" s="47">
         <v>10</v>
@@ -23693,7 +23709,7 @@
         <v>46509</v>
       </c>
       <c r="L52" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M52" s="49">
         <v>0</v>
@@ -23767,19 +23783,19 @@
     </row>
     <row r="53" spans="1:69" ht="42" customHeight="1">
       <c r="A53" s="20" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="B53" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C53" s="22" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
       <c r="D53" s="22" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
       <c r="E53" s="22" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
       <c r="F53" s="47">
         <v>14</v>
@@ -23803,7 +23819,7 @@
         <v>46516</v>
       </c>
       <c r="L53" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M53" s="49">
         <v>0</v>
@@ -23877,19 +23893,19 @@
     </row>
     <row r="54" spans="1:69" ht="42" customHeight="1">
       <c r="A54" s="20" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="B54" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C54" s="22" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
       <c r="D54" s="22" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="E54" s="22" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
       <c r="F54" s="47">
         <v>8</v>
@@ -23913,7 +23929,7 @@
         <v>46523</v>
       </c>
       <c r="L54" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M54" s="49">
         <v>0</v>
@@ -23987,19 +24003,19 @@
     </row>
     <row r="55" spans="1:69" ht="42" customHeight="1">
       <c r="A55" s="20" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="B55" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C55" s="22" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
       <c r="D55" s="22" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
       <c r="E55" s="22" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
       <c r="F55" s="47">
         <v>10</v>
@@ -24023,7 +24039,7 @@
         <v>46530</v>
       </c>
       <c r="L55" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M55" s="49">
         <v>0</v>
@@ -24097,19 +24113,19 @@
     </row>
     <row r="56" spans="1:69" ht="42" customHeight="1">
       <c r="A56" s="20" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="B56" s="38" t="s">
         <v>73</v>
       </c>
       <c r="C56" s="22" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
       <c r="D56" s="22" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
       <c r="E56" s="22" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
       <c r="F56" s="47">
         <v>4</v>
@@ -24133,7 +24149,7 @@
         <v>46530</v>
       </c>
       <c r="L56" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M56" s="49">
         <v>0</v>
@@ -24205,19 +24221,19 @@
     </row>
     <row r="57" spans="1:69" ht="42" customHeight="1">
       <c r="A57" s="20" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="B57" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C57" s="22" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
       <c r="D57" s="22" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="E57" s="22" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
       <c r="F57" s="47">
         <v>12</v>
@@ -24241,7 +24257,7 @@
         <v>46537</v>
       </c>
       <c r="L57" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M57" s="49">
         <v>0</v>
@@ -24313,19 +24329,19 @@
     </row>
     <row r="58" spans="1:69" ht="42" customHeight="1">
       <c r="A58" s="20" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
       <c r="B58" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C58" s="22" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
       <c r="D58" s="22" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
       <c r="E58" s="22" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
       <c r="F58" s="47">
         <v>10</v>
@@ -24349,7 +24365,7 @@
         <v>46544</v>
       </c>
       <c r="L58" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M58" s="49">
         <v>0</v>
@@ -24423,19 +24439,19 @@
     </row>
     <row r="59" spans="1:69" ht="42" customHeight="1">
       <c r="A59" s="20" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="B59" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C59" s="22" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="D59" s="22" t="s">
+        <v>324</v>
+      </c>
+      <c r="E59" s="22" t="s">
         <v>316</v>
-      </c>
-      <c r="E59" s="22" t="s">
-        <v>308</v>
       </c>
       <c r="F59" s="47">
         <v>10</v>
@@ -24459,7 +24475,7 @@
         <v>46551</v>
       </c>
       <c r="L59" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M59" s="49">
         <v>0</v>
@@ -24533,19 +24549,19 @@
     </row>
     <row r="60" spans="1:69" ht="42" customHeight="1">
       <c r="A60" s="20" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="B60" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C60" s="22" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="D60" s="22" t="s">
+        <v>327</v>
+      </c>
+      <c r="E60" s="22" t="s">
         <v>319</v>
-      </c>
-      <c r="E60" s="22" t="s">
-        <v>311</v>
       </c>
       <c r="F60" s="47">
         <v>10</v>
@@ -24569,7 +24585,7 @@
         <v>46551</v>
       </c>
       <c r="L60" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M60" s="49">
         <v>0</v>
@@ -24641,19 +24657,19 @@
     </row>
     <row r="61" spans="1:69" ht="42" customHeight="1">
       <c r="A61" s="20" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
       <c r="B61" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C61" s="22" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
       <c r="D61" s="22" t="s">
+        <v>330</v>
+      </c>
+      <c r="E61" s="22" t="s">
         <v>322</v>
-      </c>
-      <c r="E61" s="22" t="s">
-        <v>314</v>
       </c>
       <c r="F61" s="47">
         <v>8</v>
@@ -24677,7 +24693,7 @@
         <v>46558</v>
       </c>
       <c r="L61" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M61" s="49">
         <v>0</v>
@@ -24749,19 +24765,19 @@
     </row>
     <row r="62" spans="1:69" ht="42" customHeight="1">
       <c r="A62" s="20" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
       <c r="B62" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C62" s="22" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
       <c r="D62" s="22" t="s">
+        <v>333</v>
+      </c>
+      <c r="E62" s="22" t="s">
         <v>325</v>
-      </c>
-      <c r="E62" s="22" t="s">
-        <v>317</v>
       </c>
       <c r="F62" s="47">
         <v>6</v>
@@ -24785,7 +24801,7 @@
         <v>46565</v>
       </c>
       <c r="L62" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M62" s="49">
         <v>0</v>
@@ -24859,19 +24875,19 @@
     </row>
     <row r="63" spans="1:69" ht="42" customHeight="1">
       <c r="A63" s="20" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="B63" s="40" t="s">
         <v>76</v>
       </c>
       <c r="C63" s="22" t="s">
-        <v>327</v>
+        <v>335</v>
       </c>
       <c r="D63" s="22" t="s">
+        <v>336</v>
+      </c>
+      <c r="E63" s="22" t="s">
         <v>328</v>
-      </c>
-      <c r="E63" s="22" t="s">
-        <v>320</v>
       </c>
       <c r="F63" s="47">
         <v>4</v>
@@ -24895,7 +24911,7 @@
         <v>46565</v>
       </c>
       <c r="L63" s="47" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="M63" s="49">
         <v>0</v>
@@ -27633,6 +27649,13 @@
         <cfvo type="max"/>
         <color rgb="FF2563EB"/>
       </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF2563EB"/>
+      </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{B05FFF90-18D4-A5A7-8560-2BA14D3F5BBD}</x14:id>
@@ -27691,20 +27714,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="108" t="s">
-        <v>329</v>
-      </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
-      <c r="I1" s="108"/>
-      <c r="J1" s="108"/>
-      <c r="K1" s="108"/>
-      <c r="L1" s="108"/>
+      <c r="A1" s="127" t="s">
+        <v>337</v>
+      </c>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="127"/>
+      <c r="J1" s="127"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="127"/>
       <c r="M1" s="107"/>
       <c r="N1" s="107"/>
       <c r="O1" s="107"/>
@@ -27836,13 +27859,13 @@
     </row>
     <row r="3" spans="1:69" ht="36" customHeight="1">
       <c r="A3" s="19" t="s">
-        <v>330</v>
+        <v>338</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>331</v>
+        <v>339</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>332</v>
+        <v>340</v>
       </c>
       <c r="D3" s="19" t="s">
         <v>89</v>
@@ -27851,25 +27874,25 @@
         <v>97</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>333</v>
+        <v>341</v>
       </c>
       <c r="G3" s="19" t="s">
-        <v>334</v>
+        <v>342</v>
       </c>
       <c r="H3" s="19" t="s">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="I3" s="19" t="s">
-        <v>336</v>
+        <v>344</v>
       </c>
       <c r="J3" s="19" t="s">
-        <v>337</v>
+        <v>345</v>
       </c>
       <c r="K3" s="19" t="s">
         <v>95</v>
       </c>
       <c r="L3" s="19" t="s">
-        <v>338</v>
+        <v>346</v>
       </c>
       <c r="M3" s="1"/>
       <c r="N3" s="1"/>
@@ -27929,7 +27952,7 @@
       <c r="BP3" s="1"/>
       <c r="BQ3" s="1"/>
     </row>
-    <row r="4" spans="1:69" ht="81">
+    <row r="4" spans="1:69" ht="94.5">
       <c r="A4" s="84">
         <v>1</v>
       </c>
@@ -27942,12 +27965,12 @@
       <c r="D4" s="86">
         <v>11</v>
       </c>
-      <c r="E4" s="86">
-        <v>1.5</v>
-      </c>
-      <c r="F4" s="86">
+      <c r="E4" s="110">
+        <v>2.12</v>
+      </c>
+      <c r="F4" s="110">
         <f t="shared" ref="F4:F35" si="0">IF(E4="","",E4-D4)</f>
-        <v>-9.5</v>
+        <v>-8.879999999999999</v>
       </c>
       <c r="G4" s="86">
         <f>D4</f>
@@ -27955,20 +27978,20 @@
       </c>
       <c r="H4" s="86">
         <f>IF(E4="",0,E4)</f>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I4" s="86">
         <f t="shared" ref="I4:I35" si="1">MAX(576-G4,0)</f>
         <v>565</v>
       </c>
       <c r="J4" s="86" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="K4" s="86" t="s">
-        <v>425</v>
+        <v>166</v>
       </c>
       <c r="L4" s="87" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="M4" s="1"/>
       <c r="N4" s="1"/>
@@ -28052,17 +28075,17 @@
       </c>
       <c r="H5" s="86">
         <f t="shared" ref="H5:H36" si="3">H4+IF(E5="",0,E5)</f>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I5" s="86">
         <f t="shared" si="1"/>
         <v>554</v>
       </c>
       <c r="J5" s="86" t="s">
-        <v>339</v>
+        <v>347</v>
       </c>
       <c r="K5" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L5" s="87"/>
       <c r="M5" s="1"/>
@@ -28147,17 +28170,17 @@
       </c>
       <c r="H6" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I6" s="86">
         <f t="shared" si="1"/>
         <v>543</v>
       </c>
       <c r="J6" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K6" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L6" s="87"/>
       <c r="M6" s="1"/>
@@ -28242,17 +28265,17 @@
       </c>
       <c r="H7" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I7" s="86">
         <f t="shared" si="1"/>
         <v>532</v>
       </c>
       <c r="J7" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K7" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L7" s="87"/>
       <c r="M7" s="1"/>
@@ -28337,17 +28360,17 @@
       </c>
       <c r="H8" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I8" s="86">
         <f t="shared" si="1"/>
         <v>521</v>
       </c>
       <c r="J8" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K8" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L8" s="87"/>
       <c r="M8" s="1"/>
@@ -28432,17 +28455,17 @@
       </c>
       <c r="H9" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I9" s="86">
         <f t="shared" si="1"/>
         <v>510</v>
       </c>
       <c r="J9" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K9" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L9" s="87"/>
       <c r="M9" s="1"/>
@@ -28527,17 +28550,17 @@
       </c>
       <c r="H10" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I10" s="86">
         <f t="shared" si="1"/>
         <v>499</v>
       </c>
       <c r="J10" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K10" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L10" s="87"/>
       <c r="M10" s="1"/>
@@ -28622,17 +28645,17 @@
       </c>
       <c r="H11" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I11" s="86">
         <f t="shared" si="1"/>
         <v>488</v>
       </c>
       <c r="J11" s="86" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K11" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L11" s="87"/>
       <c r="M11" s="1"/>
@@ -28717,17 +28740,17 @@
       </c>
       <c r="H12" s="90">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I12" s="90">
         <f t="shared" si="1"/>
         <v>476</v>
       </c>
       <c r="J12" s="90" t="s">
-        <v>340</v>
+        <v>348</v>
       </c>
       <c r="K12" s="90" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L12" s="91"/>
       <c r="M12" s="1"/>
@@ -28812,17 +28835,17 @@
       </c>
       <c r="H13" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I13" s="86">
         <f t="shared" si="1"/>
         <v>465</v>
       </c>
       <c r="J13" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K13" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L13" s="87"/>
       <c r="M13" s="1"/>
@@ -28907,17 +28930,17 @@
       </c>
       <c r="H14" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I14" s="86">
         <f t="shared" si="1"/>
         <v>454</v>
       </c>
       <c r="J14" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K14" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L14" s="87"/>
       <c r="M14" s="1"/>
@@ -29002,17 +29025,17 @@
       </c>
       <c r="H15" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I15" s="86">
         <f t="shared" si="1"/>
         <v>443</v>
       </c>
       <c r="J15" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K15" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L15" s="87"/>
       <c r="M15" s="1"/>
@@ -29097,17 +29120,17 @@
       </c>
       <c r="H16" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I16" s="86">
         <f t="shared" si="1"/>
         <v>432</v>
       </c>
       <c r="J16" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K16" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L16" s="87"/>
       <c r="M16" s="1"/>
@@ -29192,17 +29215,17 @@
       </c>
       <c r="H17" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I17" s="86">
         <f t="shared" si="1"/>
         <v>421</v>
       </c>
       <c r="J17" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K17" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L17" s="87"/>
       <c r="M17" s="1"/>
@@ -29287,17 +29310,17 @@
       </c>
       <c r="H18" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I18" s="86">
         <f t="shared" si="1"/>
         <v>410</v>
       </c>
       <c r="J18" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K18" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L18" s="87"/>
       <c r="M18" s="1"/>
@@ -29382,17 +29405,17 @@
       </c>
       <c r="H19" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I19" s="86">
         <f t="shared" si="1"/>
         <v>399</v>
       </c>
       <c r="J19" s="86" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="K19" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L19" s="87"/>
       <c r="M19" s="1"/>
@@ -29477,17 +29500,17 @@
       </c>
       <c r="H20" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I20" s="86">
         <f t="shared" si="1"/>
         <v>388</v>
       </c>
       <c r="J20" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K20" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L20" s="87"/>
       <c r="M20" s="1"/>
@@ -29572,17 +29595,17 @@
       </c>
       <c r="H21" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I21" s="86">
         <f t="shared" si="1"/>
         <v>377</v>
       </c>
       <c r="J21" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K21" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L21" s="87"/>
       <c r="M21" s="1"/>
@@ -29667,17 +29690,17 @@
       </c>
       <c r="H22" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I22" s="86">
         <f t="shared" si="1"/>
         <v>366</v>
       </c>
       <c r="J22" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K22" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L22" s="87"/>
       <c r="M22" s="1"/>
@@ -29762,17 +29785,17 @@
       </c>
       <c r="H23" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I23" s="86">
         <f t="shared" si="1"/>
         <v>355</v>
       </c>
       <c r="J23" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K23" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L23" s="87"/>
       <c r="M23" s="1"/>
@@ -29857,17 +29880,17 @@
       </c>
       <c r="H24" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I24" s="86">
         <f t="shared" si="1"/>
         <v>344</v>
       </c>
       <c r="J24" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K24" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L24" s="87"/>
       <c r="M24" s="1"/>
@@ -29952,17 +29975,17 @@
       </c>
       <c r="H25" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I25" s="86">
         <f t="shared" si="1"/>
         <v>333</v>
       </c>
       <c r="J25" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K25" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L25" s="87"/>
       <c r="M25" s="1"/>
@@ -30047,17 +30070,17 @@
       </c>
       <c r="H26" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I26" s="86">
         <f t="shared" si="1"/>
         <v>322</v>
       </c>
       <c r="J26" s="86" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K26" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L26" s="87"/>
       <c r="M26" s="1"/>
@@ -30142,17 +30165,17 @@
       </c>
       <c r="H27" s="90">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I27" s="90">
         <f t="shared" si="1"/>
         <v>310</v>
       </c>
       <c r="J27" s="90" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="K27" s="90" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L27" s="91"/>
       <c r="M27" s="1"/>
@@ -30237,17 +30260,17 @@
       </c>
       <c r="H28" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I28" s="86">
         <f t="shared" si="1"/>
         <v>299</v>
       </c>
       <c r="J28" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K28" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L28" s="87"/>
       <c r="M28" s="1"/>
@@ -30332,17 +30355,17 @@
       </c>
       <c r="H29" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I29" s="86">
         <f t="shared" si="1"/>
         <v>288</v>
       </c>
       <c r="J29" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K29" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L29" s="87"/>
       <c r="M29" s="1"/>
@@ -30427,17 +30450,17 @@
       </c>
       <c r="H30" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I30" s="86">
         <f t="shared" si="1"/>
         <v>277</v>
       </c>
       <c r="J30" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K30" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L30" s="87"/>
       <c r="M30" s="1"/>
@@ -30522,17 +30545,17 @@
       </c>
       <c r="H31" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I31" s="86">
         <f t="shared" si="1"/>
         <v>266</v>
       </c>
       <c r="J31" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K31" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L31" s="87"/>
       <c r="M31" s="1"/>
@@ -30617,17 +30640,17 @@
       </c>
       <c r="H32" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I32" s="86">
         <f t="shared" si="1"/>
         <v>255</v>
       </c>
       <c r="J32" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K32" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L32" s="87"/>
       <c r="M32" s="1"/>
@@ -30712,17 +30735,17 @@
       </c>
       <c r="H33" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I33" s="86">
         <f t="shared" si="1"/>
         <v>244</v>
       </c>
       <c r="J33" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K33" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L33" s="87"/>
       <c r="M33" s="1"/>
@@ -30807,17 +30830,17 @@
       </c>
       <c r="H34" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I34" s="86">
         <f t="shared" si="1"/>
         <v>233</v>
       </c>
       <c r="J34" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K34" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L34" s="87"/>
       <c r="M34" s="1"/>
@@ -30902,17 +30925,17 @@
       </c>
       <c r="H35" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I35" s="86">
         <f t="shared" si="1"/>
         <v>222</v>
       </c>
       <c r="J35" s="86" t="s">
-        <v>343</v>
+        <v>351</v>
       </c>
       <c r="K35" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L35" s="87"/>
       <c r="M35" s="1"/>
@@ -30997,17 +31020,17 @@
       </c>
       <c r="H36" s="86">
         <f t="shared" si="3"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I36" s="86">
         <f t="shared" ref="I36:I55" si="5">MAX(576-G36,0)</f>
         <v>211</v>
       </c>
       <c r="J36" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K36" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L36" s="87"/>
       <c r="M36" s="1"/>
@@ -31092,17 +31115,17 @@
       </c>
       <c r="H37" s="86">
         <f t="shared" ref="H37:H55" si="7">H36+IF(E37="",0,E37)</f>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I37" s="86">
         <f t="shared" si="5"/>
         <v>200</v>
       </c>
       <c r="J37" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K37" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L37" s="87"/>
       <c r="M37" s="1"/>
@@ -31187,17 +31210,17 @@
       </c>
       <c r="H38" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I38" s="86">
         <f t="shared" si="5"/>
         <v>189</v>
       </c>
       <c r="J38" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K38" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L38" s="87"/>
       <c r="M38" s="1"/>
@@ -31282,17 +31305,17 @@
       </c>
       <c r="H39" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I39" s="86">
         <f t="shared" si="5"/>
         <v>178</v>
       </c>
       <c r="J39" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K39" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L39" s="87"/>
       <c r="M39" s="1"/>
@@ -31377,17 +31400,17 @@
       </c>
       <c r="H40" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I40" s="86">
         <f t="shared" si="5"/>
         <v>167</v>
       </c>
       <c r="J40" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K40" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L40" s="87"/>
       <c r="M40" s="1"/>
@@ -31472,17 +31495,17 @@
       </c>
       <c r="H41" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I41" s="86">
         <f t="shared" si="5"/>
         <v>156</v>
       </c>
       <c r="J41" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K41" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L41" s="87"/>
       <c r="M41" s="1"/>
@@ -31567,17 +31590,17 @@
       </c>
       <c r="H42" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I42" s="86">
         <f t="shared" si="5"/>
         <v>145</v>
       </c>
       <c r="J42" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K42" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L42" s="87"/>
       <c r="M42" s="1"/>
@@ -31662,17 +31685,17 @@
       </c>
       <c r="H43" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I43" s="86">
         <f t="shared" si="5"/>
         <v>134</v>
       </c>
       <c r="J43" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K43" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L43" s="87"/>
       <c r="M43" s="1"/>
@@ -31757,17 +31780,17 @@
       </c>
       <c r="H44" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I44" s="86">
         <f t="shared" si="5"/>
         <v>123</v>
       </c>
       <c r="J44" s="86" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K44" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L44" s="87"/>
       <c r="M44" s="1"/>
@@ -31852,17 +31875,17 @@
       </c>
       <c r="H45" s="90">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I45" s="90">
         <f t="shared" si="5"/>
         <v>111</v>
       </c>
       <c r="J45" s="90" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="K45" s="90" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L45" s="91"/>
       <c r="M45" s="1"/>
@@ -31947,17 +31970,17 @@
       </c>
       <c r="H46" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I46" s="86">
         <f t="shared" si="5"/>
         <v>100</v>
       </c>
       <c r="J46" s="86" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="K46" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L46" s="87"/>
       <c r="M46" s="1"/>
@@ -32042,17 +32065,17 @@
       </c>
       <c r="H47" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I47" s="86">
         <f t="shared" si="5"/>
         <v>89</v>
       </c>
       <c r="J47" s="86" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="K47" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L47" s="87"/>
       <c r="M47" s="1"/>
@@ -32137,17 +32160,17 @@
       </c>
       <c r="H48" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I48" s="86">
         <f t="shared" si="5"/>
         <v>78</v>
       </c>
       <c r="J48" s="86" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="K48" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L48" s="87"/>
       <c r="M48" s="1"/>
@@ -32232,17 +32255,17 @@
       </c>
       <c r="H49" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I49" s="86">
         <f t="shared" si="5"/>
         <v>67</v>
       </c>
       <c r="J49" s="86" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="K49" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L49" s="87"/>
       <c r="M49" s="1"/>
@@ -32327,17 +32350,17 @@
       </c>
       <c r="H50" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I50" s="86">
         <f t="shared" si="5"/>
         <v>56</v>
       </c>
       <c r="J50" s="86" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="K50" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L50" s="87"/>
       <c r="M50" s="1"/>
@@ -32422,17 +32445,17 @@
       </c>
       <c r="H51" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I51" s="86">
         <f t="shared" si="5"/>
         <v>45</v>
       </c>
       <c r="J51" s="86" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="K51" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L51" s="87"/>
       <c r="M51" s="1"/>
@@ -32517,17 +32540,17 @@
       </c>
       <c r="H52" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I52" s="86">
         <f t="shared" si="5"/>
         <v>34</v>
       </c>
       <c r="J52" s="86" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="K52" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L52" s="87"/>
       <c r="M52" s="1"/>
@@ -32612,17 +32635,17 @@
       </c>
       <c r="H53" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I53" s="86">
         <f t="shared" si="5"/>
         <v>23</v>
       </c>
       <c r="J53" s="86" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="K53" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L53" s="87"/>
       <c r="M53" s="1"/>
@@ -32707,17 +32730,17 @@
       </c>
       <c r="H54" s="86">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I54" s="86">
         <f t="shared" si="5"/>
         <v>12</v>
       </c>
       <c r="J54" s="86" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="K54" s="86" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L54" s="87"/>
       <c r="M54" s="1"/>
@@ -32802,17 +32825,17 @@
       </c>
       <c r="H55" s="90">
         <f t="shared" si="7"/>
-        <v>1.5</v>
+        <v>2.12</v>
       </c>
       <c r="I55" s="90">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="J55" s="90" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="K55" s="90" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="L55" s="91"/>
       <c r="M55" s="1"/>
@@ -36093,6 +36116,13 @@
         <cfvo type="max"/>
         <color rgb="FF2563EB"/>
       </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="9">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF2563EB"/>
+      </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
           <x14:id>{B9CF9B83-EEEF-806F-3865-A7F6C560F42A}</x14:id>
@@ -36116,6 +36146,13 @@
       </dataBar>
     </cfRule>
     <cfRule type="dataBar" priority="8">
+      <dataBar>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FF16A34A"/>
+      </dataBar>
+    </cfRule>
+    <cfRule type="dataBar" priority="10">
       <dataBar>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -36189,16 +36226,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="108" t="s">
-        <v>347</v>
-      </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
+      <c r="A1" s="127" t="s">
+        <v>355</v>
+      </c>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -36343,7 +36380,7 @@
         <v>89</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="E3" s="19" t="s">
         <v>37</v>
@@ -37080,10 +37117,10 @@
       <c r="BQ11" s="1"/>
     </row>
     <row r="12" spans="1:69" ht="15">
-      <c r="A12" s="128" t="s">
-        <v>349</v>
-      </c>
-      <c r="B12" s="129"/>
+      <c r="A12" s="131" t="s">
+        <v>357</v>
+      </c>
+      <c r="B12" s="132"/>
       <c r="C12" s="42">
         <v>576</v>
       </c>
@@ -43425,16 +43462,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="108" t="s">
-        <v>350</v>
-      </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
-      <c r="E1" s="108"/>
-      <c r="F1" s="108"/>
-      <c r="G1" s="108"/>
-      <c r="H1" s="108"/>
+      <c r="A1" s="127" t="s">
+        <v>358</v>
+      </c>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
+      <c r="E1" s="127"/>
+      <c r="F1" s="127"/>
+      <c r="G1" s="127"/>
+      <c r="H1" s="127"/>
       <c r="I1" s="107"/>
       <c r="J1" s="107"/>
       <c r="K1" s="107"/>
@@ -43569,16 +43606,16 @@
       <c r="BQ2" s="1"/>
     </row>
     <row r="3" spans="1:69" ht="15">
-      <c r="A3" s="109" t="s">
-        <v>351</v>
-      </c>
-      <c r="B3" s="109"/>
-      <c r="C3" s="109"/>
-      <c r="D3" s="109"/>
-      <c r="E3" s="109"/>
-      <c r="F3" s="109"/>
-      <c r="G3" s="109"/>
-      <c r="H3" s="109"/>
+      <c r="A3" s="126" t="s">
+        <v>359</v>
+      </c>
+      <c r="B3" s="126"/>
+      <c r="C3" s="126"/>
+      <c r="D3" s="126"/>
+      <c r="E3" s="126"/>
+      <c r="F3" s="126"/>
+      <c r="G3" s="126"/>
+      <c r="H3" s="126"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
@@ -43643,10 +43680,10 @@
     </row>
     <row r="4" spans="1:69" ht="54">
       <c r="A4" s="102" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="B4" s="103" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
@@ -43718,10 +43755,10 @@
     </row>
     <row r="5" spans="1:69" ht="54">
       <c r="A5" s="102" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="B5" s="104" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
@@ -43793,10 +43830,10 @@
     </row>
     <row r="6" spans="1:69" ht="54">
       <c r="A6" s="102" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="B6" s="104" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C6" s="1"/>
       <c r="D6" s="1"/>
@@ -43868,10 +43905,10 @@
     </row>
     <row r="7" spans="1:69" ht="135">
       <c r="A7" s="102" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="B7" s="104" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="C7" s="1"/>
       <c r="D7" s="1"/>
@@ -43943,10 +43980,10 @@
     </row>
     <row r="8" spans="1:69" ht="121.5">
       <c r="A8" s="102" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="B8" s="104" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
@@ -44018,10 +44055,10 @@
     </row>
     <row r="9" spans="1:69" ht="67.5">
       <c r="A9" s="102" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="B9" s="104" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
@@ -44093,10 +44130,10 @@
     </row>
     <row r="10" spans="1:69" ht="67.5">
       <c r="A10" s="102" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="B10" s="104" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
       <c r="C10" s="1"/>
       <c r="D10" s="1"/>
@@ -44168,10 +44205,10 @@
     </row>
     <row r="11" spans="1:69" ht="94.5">
       <c r="A11" s="102" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
       <c r="B11" s="105" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
@@ -44385,19 +44422,19 @@
     </row>
     <row r="14" spans="1:69" ht="15">
       <c r="A14" s="19" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
       <c r="C14" s="19" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="E14" s="19" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
@@ -44466,7 +44503,7 @@
     </row>
     <row r="15" spans="1:69" ht="15">
       <c r="A15" s="106" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B15" s="22">
         <v>2</v>
@@ -44475,10 +44512,10 @@
         <v>46215</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -44547,7 +44584,7 @@
     </row>
     <row r="16" spans="1:69" ht="15">
       <c r="A16" s="106" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B16" s="22">
         <v>9</v>
@@ -44556,10 +44593,10 @@
         <v>46264</v>
       </c>
       <c r="D16" s="22" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="E16" s="25" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
@@ -44628,7 +44665,7 @@
     </row>
     <row r="17" spans="1:69" ht="15">
       <c r="A17" s="106" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="B17" s="22">
         <v>16</v>
@@ -44637,10 +44674,10 @@
         <v>46313</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
@@ -44709,7 +44746,7 @@
     </row>
     <row r="18" spans="1:69" ht="15">
       <c r="A18" s="106" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
       <c r="B18" s="22">
         <v>24</v>
@@ -44718,10 +44755,10 @@
         <v>46369</v>
       </c>
       <c r="D18" s="22" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
       <c r="E18" s="25" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
@@ -44790,7 +44827,7 @@
     </row>
     <row r="19" spans="1:69" ht="15">
       <c r="A19" s="106" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
       <c r="B19" s="22">
         <v>32</v>
@@ -44799,10 +44836,10 @@
         <v>46425</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
@@ -44871,7 +44908,7 @@
     </row>
     <row r="20" spans="1:69" ht="15">
       <c r="A20" s="106" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
       <c r="B20" s="22">
         <v>42</v>
@@ -44880,10 +44917,10 @@
         <v>46495</v>
       </c>
       <c r="D20" s="22" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
@@ -44952,7 +44989,7 @@
     </row>
     <row r="21" spans="1:69" ht="15">
       <c r="A21" s="106" t="s">
-        <v>391</v>
+        <v>399</v>
       </c>
       <c r="B21" s="22">
         <v>47</v>
@@ -44961,10 +44998,10 @@
         <v>46530</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>392</v>
+        <v>400</v>
       </c>
       <c r="E21" s="25" t="s">
-        <v>393</v>
+        <v>401</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
@@ -45033,7 +45070,7 @@
     </row>
     <row r="22" spans="1:69" ht="15">
       <c r="A22" s="106" t="s">
-        <v>394</v>
+        <v>402</v>
       </c>
       <c r="B22" s="22">
         <v>52</v>
@@ -45042,10 +45079,10 @@
         <v>46565</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>395</v>
+        <v>403</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>396</v>
+        <v>404</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -45326,16 +45363,16 @@
       <c r="BQ25" s="1"/>
     </row>
     <row r="26" spans="1:69" ht="15">
-      <c r="A26" s="109" t="s">
-        <v>397</v>
-      </c>
-      <c r="B26" s="109"/>
-      <c r="C26" s="109"/>
-      <c r="D26" s="109"/>
-      <c r="E26" s="109"/>
-      <c r="F26" s="109"/>
-      <c r="G26" s="109"/>
-      <c r="H26" s="109"/>
+      <c r="A26" s="126" t="s">
+        <v>405</v>
+      </c>
+      <c r="B26" s="126"/>
+      <c r="C26" s="126"/>
+      <c r="D26" s="126"/>
+      <c r="E26" s="126"/>
+      <c r="F26" s="126"/>
+      <c r="G26" s="126"/>
+      <c r="H26" s="126"/>
       <c r="I26" s="1"/>
       <c r="J26" s="1"/>
       <c r="K26" s="1"/>
@@ -45399,16 +45436,16 @@
       <c r="BQ26" s="1"/>
     </row>
     <row r="27" spans="1:69" ht="15">
-      <c r="A27" s="116" t="s">
-        <v>398</v>
-      </c>
-      <c r="B27" s="117"/>
-      <c r="C27" s="117"/>
-      <c r="D27" s="117"/>
-      <c r="E27" s="117"/>
-      <c r="F27" s="117"/>
-      <c r="G27" s="117"/>
-      <c r="H27" s="118"/>
+      <c r="A27" s="111" t="s">
+        <v>406</v>
+      </c>
+      <c r="B27" s="112"/>
+      <c r="C27" s="112"/>
+      <c r="D27" s="112"/>
+      <c r="E27" s="112"/>
+      <c r="F27" s="112"/>
+      <c r="G27" s="112"/>
+      <c r="H27" s="113"/>
       <c r="I27" s="1"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
@@ -45472,14 +45509,14 @@
       <c r="BQ27" s="1"/>
     </row>
     <row r="28" spans="1:69" ht="15">
-      <c r="A28" s="119"/>
-      <c r="B28" s="120"/>
-      <c r="C28" s="120"/>
-      <c r="D28" s="120"/>
-      <c r="E28" s="120"/>
-      <c r="F28" s="120"/>
-      <c r="G28" s="120"/>
-      <c r="H28" s="121"/>
+      <c r="A28" s="114"/>
+      <c r="B28" s="115"/>
+      <c r="C28" s="115"/>
+      <c r="D28" s="115"/>
+      <c r="E28" s="115"/>
+      <c r="F28" s="115"/>
+      <c r="G28" s="115"/>
+      <c r="H28" s="116"/>
       <c r="I28" s="1"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
@@ -45543,14 +45580,14 @@
       <c r="BQ28" s="1"/>
     </row>
     <row r="29" spans="1:69" ht="15">
-      <c r="A29" s="119"/>
-      <c r="B29" s="120"/>
-      <c r="C29" s="120"/>
-      <c r="D29" s="120"/>
-      <c r="E29" s="120"/>
-      <c r="F29" s="120"/>
-      <c r="G29" s="120"/>
-      <c r="H29" s="121"/>
+      <c r="A29" s="114"/>
+      <c r="B29" s="115"/>
+      <c r="C29" s="115"/>
+      <c r="D29" s="115"/>
+      <c r="E29" s="115"/>
+      <c r="F29" s="115"/>
+      <c r="G29" s="115"/>
+      <c r="H29" s="116"/>
       <c r="I29" s="1"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
@@ -45614,14 +45651,14 @@
       <c r="BQ29" s="1"/>
     </row>
     <row r="30" spans="1:69" ht="15">
-      <c r="A30" s="122"/>
-      <c r="B30" s="123"/>
-      <c r="C30" s="123"/>
-      <c r="D30" s="123"/>
-      <c r="E30" s="123"/>
-      <c r="F30" s="123"/>
-      <c r="G30" s="123"/>
-      <c r="H30" s="124"/>
+      <c r="A30" s="117"/>
+      <c r="B30" s="118"/>
+      <c r="C30" s="118"/>
+      <c r="D30" s="118"/>
+      <c r="E30" s="118"/>
+      <c r="F30" s="118"/>
+      <c r="G30" s="118"/>
+      <c r="H30" s="119"/>
       <c r="I30" s="1"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
@@ -50677,12 +50714,12 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:69" ht="21">
-      <c r="A1" s="108" t="s">
-        <v>399</v>
-      </c>
-      <c r="B1" s="108"/>
-      <c r="C1" s="108"/>
-      <c r="D1" s="108"/>
+      <c r="A1" s="127" t="s">
+        <v>407</v>
+      </c>
+      <c r="B1" s="127"/>
+      <c r="C1" s="127"/>
+      <c r="D1" s="127"/>
       <c r="E1" s="107"/>
       <c r="F1" s="107"/>
       <c r="G1" s="107"/>
@@ -50822,16 +50859,16 @@
     </row>
     <row r="3" spans="1:69" ht="15">
       <c r="A3" s="19" t="s">
-        <v>400</v>
+        <v>408</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>401</v>
+        <v>409</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>402</v>
+        <v>410</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>403</v>
+        <v>411</v>
       </c>
       <c r="E3" s="1"/>
       <c r="F3" s="1"/>
@@ -50901,16 +50938,16 @@
     </row>
     <row r="4" spans="1:69" ht="27">
       <c r="A4" s="7" t="s">
-        <v>404</v>
+        <v>412</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>405</v>
+        <v>413</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="E4" s="1"/>
       <c r="F4" s="1"/>
@@ -50980,16 +51017,16 @@
     </row>
     <row r="5" spans="1:69" ht="40.5">
       <c r="A5" s="11" t="s">
-        <v>408</v>
+        <v>416</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>409</v>
+        <v>417</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -51059,16 +51096,16 @@
     </row>
     <row r="6" spans="1:69" ht="27">
       <c r="A6" s="11" t="s">
-        <v>410</v>
+        <v>418</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>411</v>
+        <v>419</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>413</v>
+        <v>421</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -51138,16 +51175,16 @@
     </row>
     <row r="7" spans="1:69" ht="27">
       <c r="A7" s="11" t="s">
-        <v>414</v>
+        <v>422</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>415</v>
+        <v>423</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>416</v>
+        <v>424</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -51217,16 +51254,16 @@
     </row>
     <row r="8" spans="1:69" ht="27">
       <c r="A8" s="11" t="s">
-        <v>417</v>
+        <v>425</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>418</v>
+        <v>426</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>412</v>
+        <v>420</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>419</v>
+        <v>427</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -51296,16 +51333,16 @@
     </row>
     <row r="9" spans="1:69" ht="27">
       <c r="A9" s="15" t="s">
-        <v>420</v>
+        <v>428</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>421</v>
+        <v>429</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>406</v>
+        <v>414</v>
       </c>
       <c r="D9" s="17" t="s">
-        <v>407</v>
+        <v>415</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>

</xml_diff>